<commit_message>
Time entry update: IWork_2026TimeTracking.xlsx [2026-04-07 23:58 UTC]
</commit_message>
<xml_diff>
--- a/IWork_2026TimeTracking.xlsx
+++ b/IWork_2026TimeTracking.xlsx
@@ -7296,7 +7296,9 @@
       <c r="BO9" s="10" t="n"/>
       <c r="BP9" s="10" t="n"/>
       <c r="BQ9" s="10" t="n"/>
-      <c r="BR9" s="10" t="n"/>
+      <c r="BR9" s="10" t="n">
+        <v>0.5</v>
+      </c>
       <c r="BS9" s="10" t="n">
         <v>0.5</v>
       </c>

</xml_diff>

<commit_message>
Time entry update: IWork_2026TimeTracking.xlsx [2026-04-08 00:01 UTC]
</commit_message>
<xml_diff>
--- a/IWork_2026TimeTracking.xlsx
+++ b/IWork_2026TimeTracking.xlsx
@@ -7299,9 +7299,7 @@
       <c r="BR9" s="10" t="n">
         <v>0.5</v>
       </c>
-      <c r="BS9" s="10" t="n">
-        <v>0.5</v>
-      </c>
+      <c r="BS9" s="10" t="n"/>
       <c r="BT9" s="10" t="n"/>
       <c r="BU9" s="10" t="n"/>
       <c r="BV9" s="10" t="n"/>

</xml_diff>

<commit_message>
Sync from OneDrive: IWork_2026TimeTracking.xlsx [2026-04-13 15:00 UTC]
</commit_message>
<xml_diff>
--- a/IWork_2026TimeTracking.xlsx
+++ b/IWork_2026TimeTracking.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ctbuh.sharepoint.com/sites/Staff/Shared Documents/Research/Time Tracking/2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3249" documentId="8_{9C70798D-ACD7-484D-B89B-B0D73EF76BDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B4005F65-D836-B84A-A1F6-03BA960C805F}"/>
+  <xr:revisionPtr revIDLastSave="3366" documentId="8_{9C70798D-ACD7-484D-B89B-B0D73EF76BDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EC3ED7E4-C209-7E49-BF06-20BB8713F687}"/>
   <bookViews>
-    <workbookView xWindow="3160" yWindow="600" windowWidth="26880" windowHeight="19740" xr2:uid="{0C10F557-92E5-4EB6-9E48-62A8B86D346C}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="17000" windowHeight="19740" xr2:uid="{0C10F557-92E5-4EB6-9E48-62A8B86D346C}"/>
   </bookViews>
   <sheets>
     <sheet name="Tracking" sheetId="1" r:id="rId1"/>
@@ -1006,107 +1006,107 @@
       </c>
       <c r="AM1" s="4">
         <f t="shared" si="3"/>
-        <v>5</v>
+        <v>8.5</v>
       </c>
       <c r="AN1" s="4">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="AO1" s="4">
         <f t="shared" si="3"/>
-        <v>1.5</v>
+        <v>8</v>
       </c>
       <c r="AP1" s="4">
         <f t="shared" si="3"/>
-        <v>2.5</v>
+        <v>9</v>
       </c>
       <c r="AQ1" s="4">
         <f t="shared" ref="AQ1:AZ2" si="4">SUM(AQ$7:AQ$1048576)</f>
-        <v>3.5</v>
+        <v>8</v>
       </c>
       <c r="AR1" s="21">
         <f t="shared" si="4"/>
-        <v>2.5</v>
+        <v>8</v>
       </c>
       <c r="AS1" s="4">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="AT1" s="4">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="AU1" s="4">
         <f t="shared" si="4"/>
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="AV1" s="4">
         <f t="shared" si="4"/>
-        <v>3</v>
+        <v>8.5</v>
       </c>
       <c r="AW1" s="4">
         <f t="shared" si="4"/>
-        <v>1.5</v>
+        <v>9</v>
       </c>
       <c r="AX1" s="4">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="AY1" s="4">
         <f t="shared" si="4"/>
-        <v>1.5</v>
+        <v>8</v>
       </c>
       <c r="AZ1" s="4">
         <f t="shared" si="4"/>
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="BA1" s="4">
         <f t="shared" ref="BA1:BJ2" si="5">SUM(BA$7:BA$1048576)</f>
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="BB1" s="4">
         <f t="shared" si="5"/>
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="BC1" s="4">
         <f t="shared" si="5"/>
-        <v>1.5</v>
+        <v>8</v>
       </c>
       <c r="BD1" s="4">
         <f t="shared" si="5"/>
-        <v>2.5</v>
+        <v>9</v>
       </c>
       <c r="BE1" s="4">
         <f t="shared" si="5"/>
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="BF1" s="4">
         <f t="shared" si="5"/>
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="BG1" s="4">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="BH1" s="4">
         <f t="shared" si="5"/>
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="BI1" s="4">
         <f t="shared" si="5"/>
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="BJ1" s="4">
         <f t="shared" si="5"/>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="BK1" s="4">
         <f t="shared" ref="BK1:BT2" si="6">SUM(BK$7:BK$1048576)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="BL1" s="4">
         <f t="shared" si="6"/>
-        <v>6.5</v>
+        <v>8</v>
       </c>
       <c r="BM1" s="4">
         <f t="shared" si="6"/>
@@ -1130,23 +1130,23 @@
       </c>
       <c r="BR1" s="4">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="BS1" s="4">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="BT1" s="4">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>8.25</v>
       </c>
       <c r="BU1" s="4">
         <f t="shared" ref="BU1:CD2" si="7">SUM(BU$7:BU$1048576)</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="BV1" s="4">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="BW1" s="4">
         <f t="shared" si="7"/>
@@ -2056,107 +2056,107 @@
       </c>
       <c r="AM2" s="4">
         <f t="shared" si="3"/>
-        <v>5</v>
+        <v>8.5</v>
       </c>
       <c r="AN2" s="4">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="AO2" s="4">
         <f t="shared" si="3"/>
-        <v>1.5</v>
+        <v>8</v>
       </c>
       <c r="AP2" s="4">
         <f t="shared" si="3"/>
-        <v>2.5</v>
+        <v>9</v>
       </c>
       <c r="AQ2" s="4">
         <f t="shared" si="4"/>
-        <v>3.5</v>
+        <v>8</v>
       </c>
       <c r="AR2" s="21">
         <f t="shared" si="4"/>
-        <v>2.5</v>
+        <v>8</v>
       </c>
       <c r="AS2" s="4">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="AT2" s="4">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="AU2" s="4">
         <f t="shared" si="4"/>
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="AV2" s="4">
         <f t="shared" si="4"/>
-        <v>3</v>
+        <v>8.5</v>
       </c>
       <c r="AW2" s="4">
         <f t="shared" si="4"/>
-        <v>1.5</v>
+        <v>9</v>
       </c>
       <c r="AX2" s="4">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="AY2" s="4">
         <f t="shared" si="4"/>
-        <v>1.5</v>
+        <v>8</v>
       </c>
       <c r="AZ2" s="4">
         <f t="shared" si="4"/>
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="BA2" s="4">
         <f t="shared" si="5"/>
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="BB2" s="4">
         <f t="shared" si="5"/>
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="BC2" s="4">
         <f t="shared" si="5"/>
-        <v>1.5</v>
+        <v>8</v>
       </c>
       <c r="BD2" s="4">
         <f t="shared" si="5"/>
-        <v>2.5</v>
+        <v>9</v>
       </c>
       <c r="BE2" s="4">
         <f t="shared" si="5"/>
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="BF2" s="4">
         <f t="shared" si="5"/>
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="BG2" s="4">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="BH2" s="4">
         <f t="shared" si="5"/>
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="BI2" s="4">
         <f t="shared" si="5"/>
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="BJ2" s="4">
         <f t="shared" si="5"/>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="BK2" s="4">
         <f t="shared" si="6"/>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="BL2" s="4">
         <f t="shared" si="6"/>
-        <v>6.5</v>
+        <v>8</v>
       </c>
       <c r="BM2" s="4">
         <f t="shared" si="6"/>
@@ -2180,23 +2180,23 @@
       </c>
       <c r="BR2" s="4">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="BS2" s="4">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="BT2" s="4">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>8.25</v>
       </c>
       <c r="BU2" s="4">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="BV2" s="4">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="BW2" s="4">
         <f t="shared" si="7"/>
@@ -3106,7 +3106,7 @@
       </c>
       <c r="AM3" s="4">
         <f t="shared" si="26"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="AN3" s="4">
         <f t="shared" si="26"/>
@@ -3118,7 +3118,7 @@
       </c>
       <c r="AP3" s="4">
         <f t="shared" si="26"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AQ3" s="4">
         <f t="shared" si="26"/>
@@ -3142,11 +3142,11 @@
       </c>
       <c r="AV3" s="4">
         <f t="shared" si="26"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="AW3" s="4">
         <f t="shared" si="26"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AX3" s="4">
         <f t="shared" ref="AX3:CP3" si="27">IF(AX2&gt;8,AX2-8,0)</f>
@@ -3162,7 +3162,7 @@
       </c>
       <c r="BA3" s="4">
         <f t="shared" si="27"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BB3" s="4">
         <f t="shared" si="27"/>
@@ -3174,7 +3174,7 @@
       </c>
       <c r="BD3" s="4">
         <f t="shared" si="27"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BE3" s="4">
         <f t="shared" si="27"/>
@@ -3238,7 +3238,7 @@
       </c>
       <c r="BT3" s="4">
         <f t="shared" si="27"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="BU3" s="4">
         <f t="shared" si="27"/>
@@ -6900,7 +6900,7 @@
       </c>
       <c r="B7" s="17">
         <f>SUM(B8:B24)</f>
-        <v>230</v>
+        <v>316</v>
       </c>
       <c r="C7" s="9"/>
       <c r="D7" s="9"/>
@@ -7442,7 +7442,7 @@
       </c>
       <c r="B9" s="9">
         <f t="shared" ref="B9:B82" si="576">SUM($C9:$XFD9)</f>
-        <v>29</v>
+        <v>34.5</v>
       </c>
       <c r="C9" s="9"/>
       <c r="D9" s="9"/>
@@ -7504,10 +7504,14 @@
       <c r="AL9" s="10">
         <v>1</v>
       </c>
-      <c r="AM9" s="10"/>
+      <c r="AM9" s="10">
+        <v>0.5</v>
+      </c>
       <c r="AN9" s="10"/>
       <c r="AO9" s="10"/>
-      <c r="AP9" s="10"/>
+      <c r="AP9" s="10">
+        <v>1</v>
+      </c>
       <c r="AQ9" s="10">
         <v>1.5</v>
       </c>
@@ -7530,8 +7534,12 @@
       <c r="BD9" s="10">
         <v>2.5</v>
       </c>
-      <c r="BE9" s="10"/>
-      <c r="BF9" s="10"/>
+      <c r="BE9" s="10">
+        <v>1</v>
+      </c>
+      <c r="BF9" s="10">
+        <v>1</v>
+      </c>
       <c r="BG9" s="10"/>
       <c r="BH9" s="10"/>
       <c r="BI9" s="10"/>
@@ -7554,10 +7562,14 @@
       <c r="BP9" s="10"/>
       <c r="BQ9" s="10"/>
       <c r="BR9" s="10"/>
-      <c r="BS9" s="10"/>
+      <c r="BS9" s="10">
+        <v>0.5</v>
+      </c>
       <c r="BT9" s="10"/>
       <c r="BU9" s="10"/>
-      <c r="BV9" s="10"/>
+      <c r="BV9" s="10">
+        <v>1.5</v>
+      </c>
       <c r="BW9" s="10"/>
       <c r="BX9" s="10"/>
       <c r="BY9" s="10"/>
@@ -8024,7 +8036,7 @@
       </c>
       <c r="B11" s="9">
         <f t="shared" si="576"/>
-        <v>28.5</v>
+        <v>31</v>
       </c>
       <c r="C11" s="9"/>
       <c r="D11" s="9"/>
@@ -8099,10 +8111,14 @@
         <v>1</v>
       </c>
       <c r="AO11" s="10"/>
-      <c r="AP11" s="10"/>
+      <c r="AP11" s="10">
+        <v>0.5</v>
+      </c>
       <c r="AQ11" s="10"/>
       <c r="AR11" s="25"/>
-      <c r="AS11" s="10"/>
+      <c r="AS11" s="10">
+        <v>0.5</v>
+      </c>
       <c r="AT11" s="10"/>
       <c r="AU11" s="10"/>
       <c r="AV11" s="10"/>
@@ -8135,7 +8151,9 @@
       <c r="BO11" s="10"/>
       <c r="BP11" s="10"/>
       <c r="BQ11" s="10"/>
-      <c r="BR11" s="10"/>
+      <c r="BR11" s="10">
+        <v>1.5</v>
+      </c>
       <c r="BS11" s="10"/>
       <c r="BT11" s="10"/>
       <c r="BU11" s="10"/>
@@ -8336,7 +8354,7 @@
       </c>
       <c r="B12" s="9">
         <f t="shared" si="576"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C12" s="9"/>
       <c r="D12" s="9"/>
@@ -8375,8 +8393,12 @@
       <c r="AK12" s="10"/>
       <c r="AL12" s="10"/>
       <c r="AM12" s="10"/>
-      <c r="AN12" s="10"/>
-      <c r="AO12" s="10"/>
+      <c r="AN12" s="10">
+        <v>0.5</v>
+      </c>
+      <c r="AO12" s="10">
+        <v>0.5</v>
+      </c>
       <c r="AP12" s="10"/>
       <c r="AQ12" s="10"/>
       <c r="AR12" s="25"/>
@@ -8407,7 +8429,9 @@
       <c r="BQ12" s="10"/>
       <c r="BR12" s="10"/>
       <c r="BS12" s="10"/>
-      <c r="BT12" s="10"/>
+      <c r="BT12" s="10">
+        <v>1</v>
+      </c>
       <c r="BU12" s="10"/>
       <c r="BV12" s="10"/>
       <c r="BW12" s="10"/>
@@ -9456,7 +9480,7 @@
       </c>
       <c r="B16" s="9">
         <f t="shared" si="576"/>
-        <v>43</v>
+        <v>47.5</v>
       </c>
       <c r="C16" s="9"/>
       <c r="D16" s="9"/>
@@ -9535,8 +9559,12 @@
       </c>
       <c r="AN16" s="10"/>
       <c r="AO16" s="10"/>
-      <c r="AP16" s="10"/>
-      <c r="AQ16" s="10"/>
+      <c r="AP16" s="10">
+        <v>2</v>
+      </c>
+      <c r="AQ16" s="10">
+        <v>1</v>
+      </c>
       <c r="AR16" s="25">
         <v>1</v>
       </c>
@@ -9570,8 +9598,12 @@
       <c r="BR16" s="10"/>
       <c r="BS16" s="10"/>
       <c r="BT16" s="10"/>
-      <c r="BU16" s="10"/>
-      <c r="BV16" s="10"/>
+      <c r="BU16" s="10">
+        <v>1</v>
+      </c>
+      <c r="BV16" s="10">
+        <v>0.5</v>
+      </c>
       <c r="BW16" s="10"/>
       <c r="BX16" s="10"/>
       <c r="BY16" s="10"/>
@@ -10308,7 +10340,7 @@
       </c>
       <c r="B19" s="9">
         <f t="shared" si="576"/>
-        <v>42.5</v>
+        <v>103</v>
       </c>
       <c r="C19" s="9"/>
       <c r="D19" s="9"/>
@@ -10370,30 +10402,60 @@
       <c r="AJ19" s="10"/>
       <c r="AK19" s="10"/>
       <c r="AL19" s="10"/>
-      <c r="AM19" s="10"/>
-      <c r="AN19" s="10"/>
-      <c r="AO19" s="10"/>
+      <c r="AM19" s="10">
+        <v>3</v>
+      </c>
+      <c r="AN19" s="10">
+        <v>3.5</v>
+      </c>
+      <c r="AO19" s="10">
+        <v>3.5</v>
+      </c>
       <c r="AP19" s="10">
+        <v>3</v>
+      </c>
+      <c r="AQ19" s="10">
+        <v>4</v>
+      </c>
+      <c r="AR19" s="25">
+        <v>3</v>
+      </c>
+      <c r="AS19" s="10">
+        <v>2.5</v>
+      </c>
+      <c r="AT19" s="10">
+        <v>2</v>
+      </c>
+      <c r="AU19" s="10">
+        <v>3</v>
+      </c>
+      <c r="AV19" s="10">
+        <v>3</v>
+      </c>
+      <c r="AW19" s="10">
+        <v>2.5</v>
+      </c>
+      <c r="AX19" s="10">
+        <v>3</v>
+      </c>
+      <c r="AY19" s="10">
         <v>1</v>
       </c>
-      <c r="AQ19" s="10">
+      <c r="AZ19" s="10">
+        <v>0.5</v>
+      </c>
+      <c r="BA19" s="10">
+        <v>5</v>
+      </c>
+      <c r="BB19" s="10">
+        <v>4</v>
+      </c>
+      <c r="BC19" s="10">
+        <v>4</v>
+      </c>
+      <c r="BD19" s="10">
         <v>2</v>
       </c>
-      <c r="AR19" s="25">
-        <v>1</v>
-      </c>
-      <c r="AS19" s="10"/>
-      <c r="AT19" s="10"/>
-      <c r="AU19" s="10"/>
-      <c r="AV19" s="10"/>
-      <c r="AW19" s="10"/>
-      <c r="AX19" s="10"/>
-      <c r="AY19" s="10"/>
-      <c r="AZ19" s="10"/>
-      <c r="BA19" s="10"/>
-      <c r="BB19" s="10"/>
-      <c r="BC19" s="10"/>
-      <c r="BD19" s="10"/>
       <c r="BE19" s="10"/>
       <c r="BF19" s="10"/>
       <c r="BG19" s="10"/>
@@ -10407,11 +10469,21 @@
       <c r="BO19" s="10"/>
       <c r="BP19" s="10"/>
       <c r="BQ19" s="10"/>
-      <c r="BR19" s="10"/>
-      <c r="BS19" s="10"/>
-      <c r="BT19" s="10"/>
-      <c r="BU19" s="10"/>
-      <c r="BV19" s="10"/>
+      <c r="BR19" s="10">
+        <v>1</v>
+      </c>
+      <c r="BS19" s="10">
+        <v>2</v>
+      </c>
+      <c r="BT19" s="10">
+        <v>3</v>
+      </c>
+      <c r="BU19" s="10">
+        <v>3</v>
+      </c>
+      <c r="BV19" s="10">
+        <v>3</v>
+      </c>
       <c r="BW19" s="10"/>
       <c r="BX19" s="10"/>
       <c r="BY19" s="10"/>
@@ -10608,7 +10680,7 @@
       </c>
       <c r="B20" s="9">
         <f t="shared" si="576"/>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C20" s="9"/>
       <c r="D20" s="9"/>
@@ -10652,10 +10724,18 @@
       <c r="AP20" s="10"/>
       <c r="AQ20" s="10"/>
       <c r="AR20" s="25"/>
-      <c r="AS20" s="10"/>
-      <c r="AT20" s="10"/>
-      <c r="AU20" s="10"/>
-      <c r="AV20" s="10"/>
+      <c r="AS20" s="10">
+        <v>0.5</v>
+      </c>
+      <c r="AT20" s="10">
+        <v>1</v>
+      </c>
+      <c r="AU20" s="10">
+        <v>1</v>
+      </c>
+      <c r="AV20" s="10">
+        <v>0.5</v>
+      </c>
       <c r="AW20" s="10"/>
       <c r="AX20" s="10"/>
       <c r="AY20" s="10"/>
@@ -11688,7 +11768,7 @@
       </c>
       <c r="B24" s="9">
         <f t="shared" si="576"/>
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="C24" s="9"/>
       <c r="D24" s="9"/>
@@ -11737,7 +11817,9 @@
       <c r="AM24" s="10">
         <v>1</v>
       </c>
-      <c r="AN24" s="10"/>
+      <c r="AN24" s="10">
+        <v>1</v>
+      </c>
       <c r="AO24" s="10"/>
       <c r="AP24" s="10"/>
       <c r="AQ24" s="10"/>
@@ -11756,10 +11838,14 @@
       <c r="BD24" s="10"/>
       <c r="BE24" s="10"/>
       <c r="BF24" s="10"/>
-      <c r="BG24" s="10"/>
-      <c r="BH24" s="10"/>
+      <c r="BG24" s="10">
+        <v>3</v>
+      </c>
+      <c r="BH24" s="10">
+        <v>3</v>
+      </c>
       <c r="BI24" s="10">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="BJ24" s="10">
         <v>6</v>
@@ -13864,7 +13950,7 @@
       </c>
       <c r="B32" s="9">
         <f t="shared" si="576"/>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C32" s="9"/>
       <c r="D32" s="9"/>
@@ -13920,10 +14006,18 @@
       <c r="BB32" s="10"/>
       <c r="BC32" s="10"/>
       <c r="BD32" s="10"/>
-      <c r="BE32" s="10"/>
-      <c r="BF32" s="10"/>
-      <c r="BG32" s="10"/>
-      <c r="BH32" s="10"/>
+      <c r="BE32" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="BF32" s="10">
+        <v>0.5</v>
+      </c>
+      <c r="BG32" s="10">
+        <v>2</v>
+      </c>
+      <c r="BH32" s="10">
+        <v>1</v>
+      </c>
       <c r="BI32" s="10"/>
       <c r="BJ32" s="10"/>
       <c r="BK32" s="10"/>
@@ -16831,7 +16925,7 @@
       </c>
       <c r="B43" s="9">
         <f t="shared" si="576"/>
-        <v>2.5</v>
+        <v>4.5</v>
       </c>
       <c r="C43" s="9"/>
       <c r="D43" s="9"/>
@@ -16872,7 +16966,9 @@
       <c r="AK43" s="10"/>
       <c r="AL43" s="10"/>
       <c r="AM43" s="10"/>
-      <c r="AN43" s="10"/>
+      <c r="AN43" s="10">
+        <v>2</v>
+      </c>
       <c r="AO43" s="10"/>
       <c r="AP43" s="10"/>
       <c r="AQ43" s="10"/>
@@ -17377,7 +17473,7 @@
       </c>
       <c r="B45" s="9">
         <f t="shared" si="576"/>
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="C45" s="9"/>
       <c r="D45" s="9"/>
@@ -17435,7 +17531,9 @@
         <v>2</v>
       </c>
       <c r="AN45" s="10"/>
-      <c r="AO45" s="10"/>
+      <c r="AO45" s="10">
+        <v>0.5</v>
+      </c>
       <c r="AP45" s="10"/>
       <c r="AQ45" s="10"/>
       <c r="AR45" s="25"/>
@@ -17443,9 +17541,15 @@
       <c r="AT45" s="10"/>
       <c r="AU45" s="10"/>
       <c r="AV45" s="10"/>
-      <c r="AW45" s="10"/>
-      <c r="AX45" s="10"/>
-      <c r="AY45" s="10"/>
+      <c r="AW45" s="10">
+        <v>2</v>
+      </c>
+      <c r="AX45" s="10">
+        <v>1</v>
+      </c>
+      <c r="AY45" s="10">
+        <v>0.5</v>
+      </c>
       <c r="AZ45" s="10"/>
       <c r="BA45" s="10"/>
       <c r="BB45" s="10"/>
@@ -17665,7 +17769,7 @@
       </c>
       <c r="B46" s="9">
         <f t="shared" si="576"/>
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="C46" s="9"/>
       <c r="D46" s="9"/>
@@ -17705,22 +17809,54 @@
       <c r="AL46" s="10"/>
       <c r="AM46" s="10"/>
       <c r="AN46" s="10"/>
-      <c r="AO46" s="10"/>
-      <c r="AP46" s="10"/>
-      <c r="AQ46" s="10"/>
-      <c r="AR46" s="25"/>
-      <c r="AS46" s="10"/>
-      <c r="AT46" s="10"/>
-      <c r="AU46" s="10"/>
-      <c r="AV46" s="10"/>
-      <c r="AW46" s="10"/>
-      <c r="AX46" s="10"/>
-      <c r="AY46" s="10"/>
-      <c r="AZ46" s="10"/>
-      <c r="BA46" s="10"/>
-      <c r="BB46" s="10"/>
-      <c r="BC46" s="10"/>
-      <c r="BD46" s="10"/>
+      <c r="AO46" s="10">
+        <v>2</v>
+      </c>
+      <c r="AP46" s="10">
+        <v>1</v>
+      </c>
+      <c r="AQ46" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="AR46" s="25">
+        <v>3.5</v>
+      </c>
+      <c r="AS46" s="10">
+        <v>4.5</v>
+      </c>
+      <c r="AT46" s="10">
+        <v>3</v>
+      </c>
+      <c r="AU46" s="10">
+        <v>1</v>
+      </c>
+      <c r="AV46" s="10">
+        <v>2</v>
+      </c>
+      <c r="AW46" s="10">
+        <v>3</v>
+      </c>
+      <c r="AX46" s="10">
+        <v>2</v>
+      </c>
+      <c r="AY46" s="10">
+        <v>2</v>
+      </c>
+      <c r="AZ46" s="10">
+        <v>2.5</v>
+      </c>
+      <c r="BA46" s="10">
+        <v>3</v>
+      </c>
+      <c r="BB46" s="10">
+        <v>2</v>
+      </c>
+      <c r="BC46" s="10">
+        <v>2.5</v>
+      </c>
+      <c r="BD46" s="10">
+        <v>3</v>
+      </c>
       <c r="BE46" s="10"/>
       <c r="BF46" s="10"/>
       <c r="BG46" s="10"/>
@@ -17737,8 +17873,12 @@
       <c r="BR46" s="10"/>
       <c r="BS46" s="10"/>
       <c r="BT46" s="10"/>
-      <c r="BU46" s="10"/>
-      <c r="BV46" s="10"/>
+      <c r="BU46" s="10">
+        <v>1</v>
+      </c>
+      <c r="BV46" s="10">
+        <v>0.5</v>
+      </c>
       <c r="BW46" s="10"/>
       <c r="BX46" s="10"/>
       <c r="BY46" s="10"/>
@@ -18757,7 +18897,7 @@
       </c>
       <c r="B50" s="9">
         <f t="shared" si="576"/>
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="C50" s="9"/>
       <c r="D50" s="9"/>
@@ -18823,22 +18963,40 @@
       <c r="AQ50" s="10"/>
       <c r="AR50" s="25"/>
       <c r="AS50" s="10"/>
-      <c r="AT50" s="10"/>
+      <c r="AT50" s="10">
+        <v>1.5</v>
+      </c>
       <c r="AU50" s="10"/>
       <c r="AV50" s="10"/>
       <c r="AW50" s="10"/>
-      <c r="AX50" s="10"/>
-      <c r="AY50" s="10"/>
-      <c r="AZ50" s="10"/>
+      <c r="AX50" s="10">
+        <v>0.5</v>
+      </c>
+      <c r="AY50" s="10">
+        <v>2.5</v>
+      </c>
+      <c r="AZ50" s="10">
+        <v>1.5</v>
+      </c>
       <c r="BA50" s="10"/>
       <c r="BB50" s="10"/>
       <c r="BC50" s="10"/>
       <c r="BD50" s="10"/>
-      <c r="BE50" s="10"/>
-      <c r="BF50" s="10"/>
-      <c r="BG50" s="10"/>
-      <c r="BH50" s="10"/>
-      <c r="BI50" s="10"/>
+      <c r="BE50" s="10">
+        <v>1</v>
+      </c>
+      <c r="BF50" s="10">
+        <v>2</v>
+      </c>
+      <c r="BG50" s="10">
+        <v>3</v>
+      </c>
+      <c r="BH50" s="10">
+        <v>3</v>
+      </c>
+      <c r="BI50" s="10">
+        <v>2</v>
+      </c>
       <c r="BJ50" s="10"/>
       <c r="BK50" s="10"/>
       <c r="BL50" s="10"/>
@@ -18847,8 +19005,12 @@
       <c r="BO50" s="10"/>
       <c r="BP50" s="10"/>
       <c r="BQ50" s="10"/>
-      <c r="BR50" s="10"/>
-      <c r="BS50" s="10"/>
+      <c r="BR50" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="BS50" s="10">
+        <v>1.5</v>
+      </c>
       <c r="BT50" s="10"/>
       <c r="BU50" s="10"/>
       <c r="BV50" s="10"/>
@@ -23367,7 +23529,7 @@
       </c>
       <c r="B67" s="9">
         <f t="shared" si="576"/>
-        <v>0</v>
+        <v>3.5</v>
       </c>
       <c r="C67" s="9"/>
       <c r="D67" s="9"/>
@@ -23428,9 +23590,15 @@
       <c r="BG67" s="10"/>
       <c r="BH67" s="10"/>
       <c r="BI67" s="10"/>
-      <c r="BJ67" s="10"/>
-      <c r="BK67" s="10"/>
-      <c r="BL67" s="10"/>
+      <c r="BJ67" s="10">
+        <v>1</v>
+      </c>
+      <c r="BK67" s="10">
+        <v>1</v>
+      </c>
+      <c r="BL67" s="10">
+        <v>1.5</v>
+      </c>
       <c r="BM67" s="10"/>
       <c r="BN67" s="25"/>
       <c r="BO67" s="10"/>
@@ -24722,7 +24890,7 @@
       </c>
       <c r="B72" s="9">
         <f t="shared" si="576"/>
-        <v>9.5</v>
+        <v>10.5</v>
       </c>
       <c r="C72" s="9"/>
       <c r="D72" s="9"/>
@@ -24794,7 +24962,9 @@
       <c r="BF72" s="10"/>
       <c r="BG72" s="10"/>
       <c r="BH72" s="10"/>
-      <c r="BI72" s="10"/>
+      <c r="BI72" s="10">
+        <v>1</v>
+      </c>
       <c r="BJ72" s="10"/>
       <c r="BK72" s="10"/>
       <c r="BL72" s="10"/>
@@ -25004,7 +25174,7 @@
       </c>
       <c r="B73" s="9">
         <f t="shared" si="576"/>
-        <v>0</v>
+        <v>6.5</v>
       </c>
       <c r="C73" s="9"/>
       <c r="D73" s="9"/>
@@ -25074,10 +25244,18 @@
       <c r="BP73" s="10"/>
       <c r="BQ73" s="10"/>
       <c r="BR73" s="10"/>
-      <c r="BS73" s="10"/>
-      <c r="BT73" s="10"/>
-      <c r="BU73" s="10"/>
-      <c r="BV73" s="10"/>
+      <c r="BS73" s="10">
+        <v>1</v>
+      </c>
+      <c r="BT73" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="BU73" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="BV73" s="10">
+        <v>2.5</v>
+      </c>
       <c r="BW73" s="10"/>
       <c r="BX73" s="10"/>
       <c r="BY73" s="10"/>
@@ -25274,7 +25452,7 @@
       </c>
       <c r="B74" s="9">
         <f t="shared" si="576"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C74" s="9"/>
       <c r="D74" s="9"/>
@@ -25330,7 +25508,9 @@
       <c r="BB74" s="10"/>
       <c r="BC74" s="10"/>
       <c r="BD74" s="10"/>
-      <c r="BE74" s="10"/>
+      <c r="BE74" s="10">
+        <v>1.5</v>
+      </c>
       <c r="BF74" s="10"/>
       <c r="BG74" s="10"/>
       <c r="BH74" s="10"/>
@@ -25346,7 +25526,9 @@
       <c r="BR74" s="10"/>
       <c r="BS74" s="10"/>
       <c r="BT74" s="10"/>
-      <c r="BU74" s="10"/>
+      <c r="BU74" s="10">
+        <v>0.5</v>
+      </c>
       <c r="BV74" s="10"/>
       <c r="BW74" s="10"/>
       <c r="BX74" s="10"/>
@@ -26081,7 +26263,7 @@
       </c>
       <c r="B77" s="9">
         <f t="shared" si="577"/>
-        <v>8.5</v>
+        <v>9.25</v>
       </c>
       <c r="C77" s="9"/>
       <c r="D77" s="9"/>
@@ -26166,7 +26348,9 @@
       <c r="BQ77" s="10"/>
       <c r="BR77" s="10"/>
       <c r="BS77" s="10"/>
-      <c r="BT77" s="10"/>
+      <c r="BT77" s="10">
+        <v>0.75</v>
+      </c>
       <c r="BU77" s="10"/>
       <c r="BV77" s="10"/>
       <c r="BW77" s="10"/>
@@ -26365,7 +26549,7 @@
       </c>
       <c r="B78" s="9">
         <f t="shared" si="577"/>
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="C78" s="9"/>
       <c r="D78" s="9"/>
@@ -26424,19 +26608,33 @@
       <c r="AQ78" s="10"/>
       <c r="AR78" s="25"/>
       <c r="AS78" s="10"/>
-      <c r="AT78" s="10"/>
+      <c r="AT78" s="10">
+        <v>0.5</v>
+      </c>
       <c r="AU78" s="10"/>
       <c r="AV78" s="10"/>
       <c r="AW78" s="10"/>
-      <c r="AX78" s="10"/>
-      <c r="AY78" s="10"/>
-      <c r="AZ78" s="10"/>
+      <c r="AX78" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="AY78" s="10">
+        <v>0.5</v>
+      </c>
+      <c r="AZ78" s="10">
+        <v>1.5</v>
+      </c>
       <c r="BA78" s="10"/>
       <c r="BB78" s="10"/>
       <c r="BC78" s="10"/>
-      <c r="BD78" s="10"/>
-      <c r="BE78" s="10"/>
-      <c r="BF78" s="10"/>
+      <c r="BD78" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="BE78" s="10">
+        <v>2</v>
+      </c>
+      <c r="BF78" s="10">
+        <v>2.5</v>
+      </c>
       <c r="BG78" s="10"/>
       <c r="BH78" s="10"/>
       <c r="BI78" s="10"/>
@@ -26448,10 +26646,18 @@
       <c r="BO78" s="10"/>
       <c r="BP78" s="10"/>
       <c r="BQ78" s="10"/>
-      <c r="BR78" s="10"/>
-      <c r="BS78" s="10"/>
-      <c r="BT78" s="10"/>
-      <c r="BU78" s="10"/>
+      <c r="BR78" s="10">
+        <v>1</v>
+      </c>
+      <c r="BS78" s="10">
+        <v>3</v>
+      </c>
+      <c r="BT78" s="10">
+        <v>2</v>
+      </c>
+      <c r="BU78" s="10">
+        <v>1</v>
+      </c>
       <c r="BV78" s="10"/>
       <c r="BW78" s="10"/>
       <c r="BX78" s="10"/>
@@ -27767,7 +27973,7 @@
       </c>
       <c r="B83" s="9">
         <f t="shared" ref="B83:B85" si="578">SUM($C83:$XFD83)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C83" s="9"/>
       <c r="D83" s="9"/>
@@ -27836,7 +28042,9 @@
       <c r="BO83" s="10"/>
       <c r="BP83" s="10"/>
       <c r="BQ83" s="10"/>
-      <c r="BR83" s="10"/>
+      <c r="BR83" s="10">
+        <v>3</v>
+      </c>
       <c r="BS83" s="10"/>
       <c r="BT83" s="10"/>
       <c r="BU83" s="10"/>
@@ -30898,12 +31106,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="be2d32d5-45e4-45f8-8cca-e731efdae529">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -31148,20 +31358,27 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="be2d32d5-45e4-45f8-8cca-e731efdae529">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CEFE62B7-6772-44D0-ACCE-A546E807D9BB}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{035973C1-EA40-447A-BB47-72CAA2093BEE}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6"/>
+    <ds:schemaRef ds:uri="be2d32d5-45e4-45f8-8cca-e731efdae529"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -31186,18 +31403,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{035973C1-EA40-447A-BB47-72CAA2093BEE}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CEFE62B7-6772-44D0-ACCE-A546E807D9BB}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6"/>
-    <ds:schemaRef ds:uri="be2d32d5-45e4-45f8-8cca-e731efdae529"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Sync from OneDrive: IWork_2026TimeTracking.xlsx [2026-04-13 16:00 UTC]
</commit_message>
<xml_diff>
--- a/IWork_2026TimeTracking.xlsx
+++ b/IWork_2026TimeTracking.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ctbuh.sharepoint.com/sites/Staff/Shared Documents/Research/Time Tracking/2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3366" documentId="8_{9C70798D-ACD7-484D-B89B-B0D73EF76BDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EC3ED7E4-C209-7E49-BF06-20BB8713F687}"/>
+  <xr:revisionPtr revIDLastSave="3376" documentId="8_{9C70798D-ACD7-484D-B89B-B0D73EF76BDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F72D0FB9-7F90-A543-A847-0B213B36E561}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="17000" windowHeight="19740" xr2:uid="{0C10F557-92E5-4EB6-9E48-62A8B86D346C}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="17000" windowHeight="17800" xr2:uid="{0C10F557-92E5-4EB6-9E48-62A8B86D346C}"/>
   </bookViews>
   <sheets>
     <sheet name="Tracking" sheetId="1" r:id="rId1"/>
@@ -7442,7 +7442,7 @@
       </c>
       <c r="B9" s="9">
         <f t="shared" ref="B9:B82" si="576">SUM($C9:$XFD9)</f>
-        <v>34.5</v>
+        <v>73.5</v>
       </c>
       <c r="C9" s="9"/>
       <c r="D9" s="9"/>
@@ -7540,23 +7540,29 @@
       <c r="BF9" s="10">
         <v>1</v>
       </c>
-      <c r="BG9" s="10"/>
-      <c r="BH9" s="10"/>
-      <c r="BI9" s="10"/>
+      <c r="BG9" s="10">
+        <v>3</v>
+      </c>
+      <c r="BH9" s="10">
+        <v>3</v>
+      </c>
+      <c r="BI9" s="10">
+        <v>5</v>
+      </c>
       <c r="BJ9" s="10">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="BK9" s="10">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="BL9" s="10">
-        <v>0.5</v>
+        <v>6.5</v>
       </c>
       <c r="BM9" s="10">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="BN9" s="25">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="BO9" s="10"/>
       <c r="BP9" s="10"/>
@@ -11768,7 +11774,7 @@
       </c>
       <c r="B24" s="9">
         <f t="shared" si="576"/>
-        <v>65</v>
+        <v>26</v>
       </c>
       <c r="C24" s="9"/>
       <c r="D24" s="9"/>
@@ -11838,30 +11844,14 @@
       <c r="BD24" s="10"/>
       <c r="BE24" s="10"/>
       <c r="BF24" s="10"/>
-      <c r="BG24" s="10">
-        <v>3</v>
-      </c>
-      <c r="BH24" s="10">
-        <v>3</v>
-      </c>
-      <c r="BI24" s="10">
-        <v>5</v>
-      </c>
-      <c r="BJ24" s="10">
-        <v>6</v>
-      </c>
-      <c r="BK24" s="10">
-        <v>6</v>
-      </c>
-      <c r="BL24" s="10">
-        <v>6</v>
-      </c>
-      <c r="BM24" s="10">
-        <v>6</v>
-      </c>
-      <c r="BN24" s="25">
-        <v>4</v>
-      </c>
+      <c r="BG24" s="10"/>
+      <c r="BH24" s="10"/>
+      <c r="BI24" s="10"/>
+      <c r="BJ24" s="10"/>
+      <c r="BK24" s="10"/>
+      <c r="BL24" s="10"/>
+      <c r="BM24" s="10"/>
+      <c r="BN24" s="25"/>
       <c r="BO24" s="10"/>
       <c r="BP24" s="10"/>
       <c r="BQ24" s="10"/>
@@ -31117,6 +31107,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008A7894324D7C3949B4D325554D1FC6DA" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="43dd22c4a0a55be49439aa2cba9a6031">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="be2d32d5-45e4-45f8-8cca-e731efdae529" xmlns:ns3="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="67300191881baa0ec8105967d66c0489" ns2:_="" ns3:_="">
     <xsd:import namespace="be2d32d5-45e4-45f8-8cca-e731efdae529"/>
@@ -31357,33 +31356,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{035973C1-EA40-447A-BB47-72CAA2093BEE}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="be2d32d5-45e4-45f8-8cca-e731efdae529"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6"/>
-    <ds:schemaRef ds:uri="be2d32d5-45e4-45f8-8cca-e731efdae529"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CEFE62B7-6772-44D0-ACCE-A546E807D9BB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2573F739-7636-44E3-8096-AD878EAC0881}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -31400,12 +31398,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CEFE62B7-6772-44D0-ACCE-A546E807D9BB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Sync from OneDrive: IWork_2026TimeTracking.xlsx [2026-04-14 17:00 UTC]
</commit_message>
<xml_diff>
--- a/IWork_2026TimeTracking.xlsx
+++ b/IWork_2026TimeTracking.xlsx
@@ -30950,4 +30950,277 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008A7894324D7C3949B4D325554D1FC6DA" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="43dd22c4a0a55be49439aa2cba9a6031">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="be2d32d5-45e4-45f8-8cca-e731efdae529" xmlns:ns3="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="67300191881baa0ec8105967d66c0489" ns2:_="" ns3:_="">
+    <xsd:import namespace="be2d32d5-45e4-45f8-8cca-e731efdae529"/>
+    <xsd:import namespace="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="be2d32d5-45e4-45f8-8cca-e731efdae529" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="10" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="11" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="7ff297e6-98dc-4a77-8782-4199b303df17" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="17" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="20" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="21" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="22" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="23" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{433bb87c-b111-4230-a796-99831eb60517}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithUsers" ma:index="18" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="19" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="be2d32d5-45e4-45f8-8cca-e731efdae529">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{56639151-3390-4733-B174-D3A8CAA5A31E}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B2A4897-00C2-4018-B6C9-09BBD2FA97C4}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED7406AD-3D3B-4FC7-B754-42493787E5EE}"/>
 </file>
</xml_diff>

<commit_message>
Update: IWork_2026TimeTracking.xlsx [2026-04-14 21:03 UTC]
</commit_message>
<xml_diff>
--- a/IWork_2026TimeTracking.xlsx
+++ b/IWork_2026TimeTracking.xlsx
@@ -7322,7 +7322,9 @@
       <c r="BW9" s="10" t="n">
         <v>0.5</v>
       </c>
-      <c r="BX9" s="10" t="n"/>
+      <c r="BX9" s="10" t="n">
+        <v>0.5</v>
+      </c>
       <c r="BY9" s="10" t="n"/>
       <c r="BZ9" s="10" t="n"/>
       <c r="CA9" s="10" t="n"/>
@@ -7916,7 +7918,9 @@
       <c r="BW11" s="10" t="n">
         <v>1.75</v>
       </c>
-      <c r="BX11" s="10" t="n"/>
+      <c r="BX11" s="10" t="n">
+        <v>1.75</v>
+      </c>
       <c r="BY11" s="10" t="n"/>
       <c r="BZ11" s="10" t="n"/>
       <c r="CA11" s="10" t="n"/>
@@ -10260,7 +10264,9 @@
       <c r="BW19" s="10" t="n">
         <v>1.5</v>
       </c>
-      <c r="BX19" s="10" t="n"/>
+      <c r="BX19" s="10" t="n">
+        <v>1.5</v>
+      </c>
       <c r="BY19" s="10" t="n"/>
       <c r="BZ19" s="10" t="n"/>
       <c r="CA19" s="10" t="n"/>
@@ -10540,7 +10546,9 @@
       <c r="BU20" s="10" t="n"/>
       <c r="BV20" s="10" t="n"/>
       <c r="BW20" s="10" t="n"/>
-      <c r="BX20" s="10" t="n"/>
+      <c r="BX20" s="10" t="n">
+        <v>0.5</v>
+      </c>
       <c r="BY20" s="10" t="n"/>
       <c r="BZ20" s="10" t="n"/>
       <c r="CA20" s="10" t="n"/>
@@ -16819,7 +16827,9 @@
       <c r="BW43" s="10" t="n">
         <v>2.25</v>
       </c>
-      <c r="BX43" s="10" t="n"/>
+      <c r="BX43" s="10" t="n">
+        <v>1</v>
+      </c>
       <c r="BY43" s="10" t="n"/>
       <c r="BZ43" s="10" t="n"/>
       <c r="CA43" s="10" t="n"/>
@@ -23471,7 +23481,9 @@
       <c r="BU67" s="10" t="n"/>
       <c r="BV67" s="10" t="n"/>
       <c r="BW67" s="10" t="n"/>
-      <c r="BX67" s="10" t="n"/>
+      <c r="BX67" s="10" t="n">
+        <v>0.5</v>
+      </c>
       <c r="BY67" s="10" t="n"/>
       <c r="BZ67" s="10" t="n"/>
       <c r="CA67" s="10" t="n"/>
@@ -23743,7 +23755,9 @@
       <c r="BU68" s="10" t="n"/>
       <c r="BV68" s="10" t="n"/>
       <c r="BW68" s="10" t="n"/>
-      <c r="BX68" s="10" t="n"/>
+      <c r="BX68" s="10" t="n">
+        <v>1.5</v>
+      </c>
       <c r="BY68" s="10" t="n"/>
       <c r="BZ68" s="10" t="n"/>
       <c r="CA68" s="10" t="n"/>
@@ -26543,7 +26557,9 @@
       </c>
       <c r="BV78" s="10" t="n"/>
       <c r="BW78" s="10" t="n"/>
-      <c r="BX78" s="10" t="n"/>
+      <c r="BX78" s="10" t="n">
+        <v>0.75</v>
+      </c>
       <c r="BY78" s="10" t="n"/>
       <c r="BZ78" s="10" t="n"/>
       <c r="CA78" s="10" t="n"/>
@@ -30950,277 +30966,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008A7894324D7C3949B4D325554D1FC6DA" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="43dd22c4a0a55be49439aa2cba9a6031">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="be2d32d5-45e4-45f8-8cca-e731efdae529" xmlns:ns3="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="67300191881baa0ec8105967d66c0489" ns2:_="" ns3:_="">
-    <xsd:import namespace="be2d32d5-45e4-45f8-8cca-e731efdae529"/>
-    <xsd:import namespace="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="be2d32d5-45e4-45f8-8cca-e731efdae529" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="10" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="11" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="7ff297e6-98dc-4a77-8782-4199b303df17" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="17" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="20" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="21" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="22" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceBillingMetadata" ma:index="23" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{433bb87c-b111-4230-a796-99831eb60517}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithUsers" ma:index="18" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="19" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="be2d32d5-45e4-45f8-8cca-e731efdae529">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{56639151-3390-4733-B174-D3A8CAA5A31E}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B2A4897-00C2-4018-B6C9-09BBD2FA97C4}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED7406AD-3D3B-4FC7-B754-42493787E5EE}"/>
 </file>
</xml_diff>

<commit_message>
Sync from OneDrive: IWork_2026TimeTracking.xlsx [2026-04-14 23:04 UTC]
</commit_message>
<xml_diff>
--- a/IWork_2026TimeTracking.xlsx
+++ b/IWork_2026TimeTracking.xlsx
@@ -30966,4 +30966,277 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008A7894324D7C3949B4D325554D1FC6DA" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="43dd22c4a0a55be49439aa2cba9a6031">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="be2d32d5-45e4-45f8-8cca-e731efdae529" xmlns:ns3="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="67300191881baa0ec8105967d66c0489" ns2:_="" ns3:_="">
+    <xsd:import namespace="be2d32d5-45e4-45f8-8cca-e731efdae529"/>
+    <xsd:import namespace="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="be2d32d5-45e4-45f8-8cca-e731efdae529" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="10" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="11" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="7ff297e6-98dc-4a77-8782-4199b303df17" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="17" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="20" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="21" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="22" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="23" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{433bb87c-b111-4230-a796-99831eb60517}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithUsers" ma:index="18" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="19" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="be2d32d5-45e4-45f8-8cca-e731efdae529">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{730FEC4D-E561-428C-804C-DFAF0EF95951}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8143F4E5-5769-4EA6-A504-F984C2EAACCD}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2DF0D4A3-6778-4178-AB8B-989A945112F6}"/>
 </file>
</xml_diff>

<commit_message>
Update: IWork_2026TimeTracking.xlsx [2026-04-15 20:54 UTC]
</commit_message>
<xml_diff>
--- a/IWork_2026TimeTracking.xlsx
+++ b/IWork_2026TimeTracking.xlsx
@@ -7325,7 +7325,9 @@
       <c r="BX9" s="10" t="n">
         <v>0.5</v>
       </c>
-      <c r="BY9" s="10" t="n"/>
+      <c r="BY9" s="10" t="n">
+        <v>0.75</v>
+      </c>
       <c r="BZ9" s="10" t="n"/>
       <c r="CA9" s="10" t="n"/>
       <c r="CB9" s="10" t="n"/>
@@ -7921,7 +7923,9 @@
       <c r="BX11" s="10" t="n">
         <v>1.75</v>
       </c>
-      <c r="BY11" s="10" t="n"/>
+      <c r="BY11" s="10" t="n">
+        <v>0.25</v>
+      </c>
       <c r="BZ11" s="10" t="n"/>
       <c r="CA11" s="10" t="n"/>
       <c r="CB11" s="10" t="n"/>
@@ -10267,7 +10271,9 @@
       <c r="BX19" s="10" t="n">
         <v>1.5</v>
       </c>
-      <c r="BY19" s="10" t="n"/>
+      <c r="BY19" s="10" t="n">
+        <v>0.5</v>
+      </c>
       <c r="BZ19" s="10" t="n"/>
       <c r="CA19" s="10" t="n"/>
       <c r="CB19" s="10" t="n"/>
@@ -10549,7 +10555,9 @@
       <c r="BX20" s="10" t="n">
         <v>0.5</v>
       </c>
-      <c r="BY20" s="10" t="n"/>
+      <c r="BY20" s="10" t="n">
+        <v>2</v>
+      </c>
       <c r="BZ20" s="10" t="n"/>
       <c r="CA20" s="10" t="n"/>
       <c r="CB20" s="10" t="n"/>
@@ -13829,7 +13837,9 @@
         <v>1.5</v>
       </c>
       <c r="BX32" s="10" t="n"/>
-      <c r="BY32" s="10" t="n"/>
+      <c r="BY32" s="10" t="n">
+        <v>1.75</v>
+      </c>
       <c r="BZ32" s="10" t="n"/>
       <c r="CA32" s="10" t="n"/>
       <c r="CB32" s="10" t="n"/>
@@ -16830,7 +16840,9 @@
       <c r="BX43" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="BY43" s="10" t="n"/>
+      <c r="BY43" s="10" t="n">
+        <v>1.5</v>
+      </c>
       <c r="BZ43" s="10" t="n"/>
       <c r="CA43" s="10" t="n"/>
       <c r="CB43" s="10" t="n"/>
@@ -17708,7 +17720,9 @@
       </c>
       <c r="BW46" s="10" t="n"/>
       <c r="BX46" s="10" t="n"/>
-      <c r="BY46" s="10" t="n"/>
+      <c r="BY46" s="10" t="n">
+        <v>0.5</v>
+      </c>
       <c r="BZ46" s="10" t="n"/>
       <c r="CA46" s="10" t="n"/>
       <c r="CB46" s="10" t="n"/>
@@ -18853,7 +18867,9 @@
         <v>0.5</v>
       </c>
       <c r="BX50" s="10" t="n"/>
-      <c r="BY50" s="10" t="n"/>
+      <c r="BY50" s="10" t="n">
+        <v>0.5</v>
+      </c>
       <c r="BZ50" s="10" t="n"/>
       <c r="CA50" s="10" t="n"/>
       <c r="CB50" s="10" t="n"/>
@@ -21847,7 +21863,9 @@
       <c r="BV61" s="10" t="n"/>
       <c r="BW61" s="10" t="n"/>
       <c r="BX61" s="10" t="n"/>
-      <c r="BY61" s="10" t="n"/>
+      <c r="BY61" s="10" t="n">
+        <v>0.25</v>
+      </c>
       <c r="BZ61" s="10" t="n"/>
       <c r="CA61" s="10" t="n"/>
       <c r="CB61" s="10" t="n"/>
@@ -23758,7 +23776,9 @@
       <c r="BX68" s="10" t="n">
         <v>1.5</v>
       </c>
-      <c r="BY68" s="10" t="n"/>
+      <c r="BY68" s="10" t="n">
+        <v>0.25</v>
+      </c>
       <c r="BZ68" s="10" t="n"/>
       <c r="CA68" s="10" t="n"/>
       <c r="CB68" s="10" t="n"/>
@@ -26560,7 +26580,9 @@
       <c r="BX78" s="10" t="n">
         <v>0.75</v>
       </c>
-      <c r="BY78" s="10" t="n"/>
+      <c r="BY78" s="10" t="n">
+        <v>0.25</v>
+      </c>
       <c r="BZ78" s="10" t="n"/>
       <c r="CA78" s="10" t="n"/>
       <c r="CB78" s="10" t="n"/>
@@ -30966,277 +30988,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008A7894324D7C3949B4D325554D1FC6DA" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="43dd22c4a0a55be49439aa2cba9a6031">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="be2d32d5-45e4-45f8-8cca-e731efdae529" xmlns:ns3="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="67300191881baa0ec8105967d66c0489" ns2:_="" ns3:_="">
-    <xsd:import namespace="be2d32d5-45e4-45f8-8cca-e731efdae529"/>
-    <xsd:import namespace="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="be2d32d5-45e4-45f8-8cca-e731efdae529" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="10" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="11" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="7ff297e6-98dc-4a77-8782-4199b303df17" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="17" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="20" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="21" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="22" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceBillingMetadata" ma:index="23" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{433bb87c-b111-4230-a796-99831eb60517}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithUsers" ma:index="18" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="19" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="be2d32d5-45e4-45f8-8cca-e731efdae529">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{730FEC4D-E561-428C-804C-DFAF0EF95951}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8143F4E5-5769-4EA6-A504-F984C2EAACCD}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2DF0D4A3-6778-4178-AB8B-989A945112F6}"/>
 </file>
</xml_diff>

<commit_message>
Sync from OneDrive: IWork_2026TimeTracking.xlsx [2026-04-15 22:00 UTC]
</commit_message>
<xml_diff>
--- a/IWork_2026TimeTracking.xlsx
+++ b/IWork_2026TimeTracking.xlsx
@@ -30988,4 +30988,277 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008A7894324D7C3949B4D325554D1FC6DA" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="43dd22c4a0a55be49439aa2cba9a6031">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="be2d32d5-45e4-45f8-8cca-e731efdae529" xmlns:ns3="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="67300191881baa0ec8105967d66c0489" ns2:_="" ns3:_="">
+    <xsd:import namespace="be2d32d5-45e4-45f8-8cca-e731efdae529"/>
+    <xsd:import namespace="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="be2d32d5-45e4-45f8-8cca-e731efdae529" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="10" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="11" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="7ff297e6-98dc-4a77-8782-4199b303df17" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="17" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="20" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="21" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="22" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="23" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{433bb87c-b111-4230-a796-99831eb60517}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithUsers" ma:index="18" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="19" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="be2d32d5-45e4-45f8-8cca-e731efdae529">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AB09AE42-FE19-440C-A928-81C3BBAAEE36}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B8B24E73-D161-4642-8897-CEB729FB6895}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F0C7987A-18FA-4388-BD39-1EE541C2D3C7}"/>
 </file>
</xml_diff>

<commit_message>
Update: IWork_2026TimeTracking.xlsx [2026-04-16 14:52 UTC]
</commit_message>
<xml_diff>
--- a/IWork_2026TimeTracking.xlsx
+++ b/IWork_2026TimeTracking.xlsx
@@ -7328,7 +7328,9 @@
       <c r="BY9" s="10" t="n">
         <v>0.75</v>
       </c>
-      <c r="BZ9" s="10" t="n"/>
+      <c r="BZ9" s="10" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CA9" s="10" t="n"/>
       <c r="CB9" s="10" t="n"/>
       <c r="CC9" s="10" t="n"/>
@@ -10274,7 +10276,9 @@
       <c r="BY19" s="10" t="n">
         <v>0.5</v>
       </c>
-      <c r="BZ19" s="10" t="n"/>
+      <c r="BZ19" s="10" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CA19" s="10" t="n"/>
       <c r="CB19" s="10" t="n"/>
       <c r="CC19" s="10" t="n"/>
@@ -10558,7 +10562,9 @@
       <c r="BY20" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="BZ20" s="10" t="n"/>
+      <c r="BZ20" s="10" t="n">
+        <v>2.5</v>
+      </c>
       <c r="CA20" s="10" t="n"/>
       <c r="CB20" s="10" t="n"/>
       <c r="CC20" s="10" t="n"/>
@@ -13840,7 +13846,9 @@
       <c r="BY32" s="10" t="n">
         <v>1.75</v>
       </c>
-      <c r="BZ32" s="10" t="n"/>
+      <c r="BZ32" s="10" t="n">
+        <v>1</v>
+      </c>
       <c r="CA32" s="10" t="n"/>
       <c r="CB32" s="10" t="n"/>
       <c r="CC32" s="10" t="n"/>
@@ -30988,277 +30996,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008A7894324D7C3949B4D325554D1FC6DA" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="43dd22c4a0a55be49439aa2cba9a6031">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="be2d32d5-45e4-45f8-8cca-e731efdae529" xmlns:ns3="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="67300191881baa0ec8105967d66c0489" ns2:_="" ns3:_="">
-    <xsd:import namespace="be2d32d5-45e4-45f8-8cca-e731efdae529"/>
-    <xsd:import namespace="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="be2d32d5-45e4-45f8-8cca-e731efdae529" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="10" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="11" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="7ff297e6-98dc-4a77-8782-4199b303df17" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="17" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="20" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="21" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="22" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceBillingMetadata" ma:index="23" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{433bb87c-b111-4230-a796-99831eb60517}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithUsers" ma:index="18" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="19" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="be2d32d5-45e4-45f8-8cca-e731efdae529">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AB09AE42-FE19-440C-A928-81C3BBAAEE36}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B8B24E73-D161-4642-8897-CEB729FB6895}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F0C7987A-18FA-4388-BD39-1EE541C2D3C7}"/>
 </file>
</xml_diff>

<commit_message>
Update: IWork_2026TimeTracking.xlsx [2026-04-16 14:53 UTC]
</commit_message>
<xml_diff>
--- a/IWork_2026TimeTracking.xlsx
+++ b/IWork_2026TimeTracking.xlsx
@@ -26867,7 +26867,9 @@
       <c r="BW79" s="10" t="n"/>
       <c r="BX79" s="10" t="n"/>
       <c r="BY79" s="10" t="n"/>
-      <c r="BZ79" s="10" t="n"/>
+      <c r="BZ79" s="10" t="n">
+        <v>1</v>
+      </c>
       <c r="CA79" s="10" t="n"/>
       <c r="CB79" s="10" t="n"/>
       <c r="CC79" s="10" t="n"/>

</xml_diff>

<commit_message>
Update: IWork_2026TimeTracking.xlsx [2026-04-16 20:23 UTC]
</commit_message>
<xml_diff>
--- a/IWork_2026TimeTracking.xlsx
+++ b/IWork_2026TimeTracking.xlsx
@@ -10277,7 +10277,7 @@
         <v>0.5</v>
       </c>
       <c r="BZ19" s="10" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="CA19" s="10" t="n"/>
       <c r="CB19" s="10" t="n"/>
@@ -11664,7 +11664,9 @@
       <c r="BW24" s="10" t="n"/>
       <c r="BX24" s="10" t="n"/>
       <c r="BY24" s="10" t="n"/>
-      <c r="BZ24" s="10" t="n"/>
+      <c r="BZ24" s="10" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CA24" s="10" t="n"/>
       <c r="CB24" s="10" t="n"/>
       <c r="CC24" s="10" t="n"/>
@@ -13847,7 +13849,7 @@
         <v>1.75</v>
       </c>
       <c r="BZ32" s="10" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="CA32" s="10" t="n"/>
       <c r="CB32" s="10" t="n"/>
@@ -16851,7 +16853,9 @@
       <c r="BY43" s="10" t="n">
         <v>1.5</v>
       </c>
-      <c r="BZ43" s="10" t="n"/>
+      <c r="BZ43" s="10" t="n">
+        <v>1.25</v>
+      </c>
       <c r="CA43" s="10" t="n"/>
       <c r="CB43" s="10" t="n"/>
       <c r="CC43" s="10" t="n"/>
@@ -17731,7 +17735,9 @@
       <c r="BY46" s="10" t="n">
         <v>0.5</v>
       </c>
-      <c r="BZ46" s="10" t="n"/>
+      <c r="BZ46" s="10" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CA46" s="10" t="n"/>
       <c r="CB46" s="10" t="n"/>
       <c r="CC46" s="10" t="n"/>
@@ -24894,7 +24900,9 @@
       <c r="BW72" s="10" t="n"/>
       <c r="BX72" s="10" t="n"/>
       <c r="BY72" s="10" t="n"/>
-      <c r="BZ72" s="10" t="n"/>
+      <c r="BZ72" s="10" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CA72" s="10" t="n"/>
       <c r="CB72" s="10" t="n"/>
       <c r="CC72" s="10" t="n"/>

</xml_diff>

<commit_message>
Sync from OneDrive: IWork_2026TimeTracking.xlsx [2026-04-17 02:00 UTC]
</commit_message>
<xml_diff>
--- a/IWork_2026TimeTracking.xlsx
+++ b/IWork_2026TimeTracking.xlsx
@@ -31006,4 +31006,277 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008A7894324D7C3949B4D325554D1FC6DA" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="43dd22c4a0a55be49439aa2cba9a6031">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="be2d32d5-45e4-45f8-8cca-e731efdae529" xmlns:ns3="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="67300191881baa0ec8105967d66c0489" ns2:_="" ns3:_="">
+    <xsd:import namespace="be2d32d5-45e4-45f8-8cca-e731efdae529"/>
+    <xsd:import namespace="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="be2d32d5-45e4-45f8-8cca-e731efdae529" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="10" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="11" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="7ff297e6-98dc-4a77-8782-4199b303df17" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="17" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="20" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="21" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="22" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="23" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{433bb87c-b111-4230-a796-99831eb60517}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithUsers" ma:index="18" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="19" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="be2d32d5-45e4-45f8-8cca-e731efdae529">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C071E994-0E91-4020-A45A-0F18E0E6D467}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{143CB26B-FB24-4D42-99C6-CF79CACD5FAD}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1A291C3D-930A-487A-8517-6095795DBF74}"/>
 </file>
</xml_diff>

<commit_message>
Update: IWork_2026TimeTracking.xlsx [2026-04-18 20:55 UTC]
</commit_message>
<xml_diff>
--- a/IWork_2026TimeTracking.xlsx
+++ b/IWork_2026TimeTracking.xlsx
@@ -7331,7 +7331,9 @@
       <c r="BZ9" s="10" t="n">
         <v>0.5</v>
       </c>
-      <c r="CA9" s="10" t="n"/>
+      <c r="CA9" s="10" t="n">
+        <v>2</v>
+      </c>
       <c r="CB9" s="10" t="n"/>
       <c r="CC9" s="10" t="n"/>
       <c r="CD9" s="10" t="n"/>
@@ -7929,7 +7931,9 @@
         <v>0.25</v>
       </c>
       <c r="BZ11" s="10" t="n"/>
-      <c r="CA11" s="10" t="n"/>
+      <c r="CA11" s="10" t="n">
+        <v>1.25</v>
+      </c>
       <c r="CB11" s="10" t="n"/>
       <c r="CC11" s="10" t="n"/>
       <c r="CD11" s="10" t="n"/>
@@ -10565,7 +10569,9 @@
       <c r="BZ20" s="10" t="n">
         <v>2.5</v>
       </c>
-      <c r="CA20" s="10" t="n"/>
+      <c r="CA20" s="10" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CB20" s="10" t="n"/>
       <c r="CC20" s="10" t="n"/>
       <c r="CD20" s="10" t="n"/>
@@ -13851,7 +13857,9 @@
       <c r="BZ32" s="10" t="n">
         <v>1.5</v>
       </c>
-      <c r="CA32" s="10" t="n"/>
+      <c r="CA32" s="10" t="n">
+        <v>1.25</v>
+      </c>
       <c r="CB32" s="10" t="n"/>
       <c r="CC32" s="10" t="n"/>
       <c r="CD32" s="10" t="n"/>
@@ -16856,7 +16864,9 @@
       <c r="BZ43" s="10" t="n">
         <v>1.25</v>
       </c>
-      <c r="CA43" s="10" t="n"/>
+      <c r="CA43" s="10" t="n">
+        <v>1.25</v>
+      </c>
       <c r="CB43" s="10" t="n"/>
       <c r="CC43" s="10" t="n"/>
       <c r="CD43" s="10" t="n"/>
@@ -18885,7 +18895,9 @@
         <v>0.5</v>
       </c>
       <c r="BZ50" s="10" t="n"/>
-      <c r="CA50" s="10" t="n"/>
+      <c r="CA50" s="10" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CB50" s="10" t="n"/>
       <c r="CC50" s="10" t="n"/>
       <c r="CD50" s="10" t="n"/>
@@ -23518,7 +23530,9 @@
       </c>
       <c r="BY67" s="10" t="n"/>
       <c r="BZ67" s="10" t="n"/>
-      <c r="CA67" s="10" t="n"/>
+      <c r="CA67" s="10" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CB67" s="10" t="n"/>
       <c r="CC67" s="10" t="n"/>
       <c r="CD67" s="10" t="n"/>
@@ -25459,7 +25473,9 @@
       <c r="BX74" s="10" t="n"/>
       <c r="BY74" s="10" t="n"/>
       <c r="BZ74" s="10" t="n"/>
-      <c r="CA74" s="10" t="n"/>
+      <c r="CA74" s="10" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CB74" s="10" t="n"/>
       <c r="CC74" s="10" t="n"/>
       <c r="CD74" s="10" t="n"/>
@@ -26600,7 +26616,9 @@
         <v>0.25</v>
       </c>
       <c r="BZ78" s="10" t="n"/>
-      <c r="CA78" s="10" t="n"/>
+      <c r="CA78" s="10" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CB78" s="10" t="n"/>
       <c r="CC78" s="10" t="n"/>
       <c r="CD78" s="10" t="n"/>
@@ -26878,7 +26896,9 @@
       <c r="BZ79" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="CA79" s="10" t="n"/>
+      <c r="CA79" s="10" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CB79" s="10" t="n"/>
       <c r="CC79" s="10" t="n"/>
       <c r="CD79" s="10" t="n"/>
@@ -31006,277 +31026,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008A7894324D7C3949B4D325554D1FC6DA" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="43dd22c4a0a55be49439aa2cba9a6031">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="be2d32d5-45e4-45f8-8cca-e731efdae529" xmlns:ns3="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="67300191881baa0ec8105967d66c0489" ns2:_="" ns3:_="">
-    <xsd:import namespace="be2d32d5-45e4-45f8-8cca-e731efdae529"/>
-    <xsd:import namespace="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="be2d32d5-45e4-45f8-8cca-e731efdae529" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="10" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="11" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="7ff297e6-98dc-4a77-8782-4199b303df17" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="17" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="20" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="21" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="22" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceBillingMetadata" ma:index="23" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{433bb87c-b111-4230-a796-99831eb60517}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithUsers" ma:index="18" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="19" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="be2d32d5-45e4-45f8-8cca-e731efdae529">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C071E994-0E91-4020-A45A-0F18E0E6D467}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{143CB26B-FB24-4D42-99C6-CF79CACD5FAD}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1A291C3D-930A-487A-8517-6095795DBF74}"/>
 </file>
</xml_diff>

<commit_message>
Sync from OneDrive: IWork_2026TimeTracking.xlsx [2026-04-21 02:00 UTC]
</commit_message>
<xml_diff>
--- a/IWork_2026TimeTracking.xlsx
+++ b/IWork_2026TimeTracking.xlsx
@@ -31026,4 +31026,277 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008A7894324D7C3949B4D325554D1FC6DA" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="43dd22c4a0a55be49439aa2cba9a6031">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="be2d32d5-45e4-45f8-8cca-e731efdae529" xmlns:ns3="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="67300191881baa0ec8105967d66c0489" ns2:_="" ns3:_="">
+    <xsd:import namespace="be2d32d5-45e4-45f8-8cca-e731efdae529"/>
+    <xsd:import namespace="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="be2d32d5-45e4-45f8-8cca-e731efdae529" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="10" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="11" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="7ff297e6-98dc-4a77-8782-4199b303df17" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="17" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="20" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="21" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="22" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="23" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{433bb87c-b111-4230-a796-99831eb60517}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithUsers" ma:index="18" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="19" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="be2d32d5-45e4-45f8-8cca-e731efdae529">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{61F6C236-D8BF-44C7-9186-EFFB515641AA}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{833117D3-06AB-4383-8015-2F0F48E6913B}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{309EB785-FC4A-41B6-BED5-3E2ED4D78668}"/>
 </file>
</xml_diff>

<commit_message>
Update: IWork_2026TimeTracking.xlsx [2026-04-22 17:25 UTC]
</commit_message>
<xml_diff>
--- a/IWork_2026TimeTracking.xlsx
+++ b/IWork_2026TimeTracking.xlsx
@@ -7936,7 +7936,9 @@
       </c>
       <c r="CB11" s="10" t="n"/>
       <c r="CC11" s="10" t="n"/>
-      <c r="CD11" s="10" t="n"/>
+      <c r="CD11" s="10" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CE11" s="10" t="n"/>
       <c r="CF11" s="10" t="n"/>
       <c r="CG11" s="10" t="n"/>
@@ -8494,7 +8496,9 @@
       <c r="CA13" s="10" t="n"/>
       <c r="CB13" s="10" t="n"/>
       <c r="CC13" s="10" t="n"/>
-      <c r="CD13" s="10" t="n"/>
+      <c r="CD13" s="10" t="n">
+        <v>1.5</v>
+      </c>
       <c r="CE13" s="10" t="n"/>
       <c r="CF13" s="10" t="n"/>
       <c r="CG13" s="10" t="n"/>
@@ -13862,7 +13866,9 @@
       </c>
       <c r="CB32" s="10" t="n"/>
       <c r="CC32" s="10" t="n"/>
-      <c r="CD32" s="10" t="n"/>
+      <c r="CD32" s="10" t="n">
+        <v>0.75</v>
+      </c>
       <c r="CE32" s="10" t="n"/>
       <c r="CF32" s="10" t="n"/>
       <c r="CG32" s="10" t="n"/>
@@ -16869,7 +16875,9 @@
       </c>
       <c r="CB43" s="10" t="n"/>
       <c r="CC43" s="10" t="n"/>
-      <c r="CD43" s="10" t="n"/>
+      <c r="CD43" s="10" t="n">
+        <v>1.75</v>
+      </c>
       <c r="CE43" s="10" t="n"/>
       <c r="CF43" s="10" t="n"/>
       <c r="CG43" s="10" t="n"/>
@@ -17751,7 +17759,9 @@
       <c r="CA46" s="10" t="n"/>
       <c r="CB46" s="10" t="n"/>
       <c r="CC46" s="10" t="n"/>
-      <c r="CD46" s="10" t="n"/>
+      <c r="CD46" s="10" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CE46" s="10" t="n"/>
       <c r="CF46" s="10" t="n"/>
       <c r="CG46" s="10" t="n"/>
@@ -18900,7 +18910,9 @@
       </c>
       <c r="CB50" s="10" t="n"/>
       <c r="CC50" s="10" t="n"/>
-      <c r="CD50" s="10" t="n"/>
+      <c r="CD50" s="10" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CE50" s="10" t="n"/>
       <c r="CF50" s="10" t="n"/>
       <c r="CG50" s="10" t="n"/>
@@ -20265,7 +20277,9 @@
       <c r="CA55" s="10" t="n"/>
       <c r="CB55" s="10" t="n"/>
       <c r="CC55" s="10" t="n"/>
-      <c r="CD55" s="10" t="n"/>
+      <c r="CD55" s="10" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CE55" s="10" t="n"/>
       <c r="CF55" s="10" t="n"/>
       <c r="CG55" s="10" t="n"/>
@@ -21896,7 +21910,9 @@
       <c r="CA61" s="10" t="n"/>
       <c r="CB61" s="10" t="n"/>
       <c r="CC61" s="10" t="n"/>
-      <c r="CD61" s="10" t="n"/>
+      <c r="CD61" s="10" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CE61" s="10" t="n"/>
       <c r="CF61" s="10" t="n"/>
       <c r="CG61" s="10" t="n"/>
@@ -22981,7 +22997,9 @@
       <c r="CA65" s="13" t="n"/>
       <c r="CB65" s="13" t="n"/>
       <c r="CC65" s="13" t="n"/>
-      <c r="CD65" s="13" t="n"/>
+      <c r="CD65" s="13" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CE65" s="13" t="n"/>
       <c r="CF65" s="13" t="n"/>
       <c r="CG65" s="13" t="n"/>
@@ -23811,7 +23829,9 @@
       <c r="CA68" s="10" t="n"/>
       <c r="CB68" s="10" t="n"/>
       <c r="CC68" s="10" t="n"/>
-      <c r="CD68" s="10" t="n"/>
+      <c r="CD68" s="10" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CE68" s="10" t="n"/>
       <c r="CF68" s="10" t="n"/>
       <c r="CG68" s="10" t="n"/>
@@ -24920,7 +24940,9 @@
       <c r="CA72" s="10" t="n"/>
       <c r="CB72" s="10" t="n"/>
       <c r="CC72" s="10" t="n"/>
-      <c r="CD72" s="10" t="n"/>
+      <c r="CD72" s="10" t="n">
+        <v>0.75</v>
+      </c>
       <c r="CE72" s="10" t="n"/>
       <c r="CF72" s="10" t="n"/>
       <c r="CG72" s="10" t="n"/>
@@ -26621,7 +26643,9 @@
       </c>
       <c r="CB78" s="10" t="n"/>
       <c r="CC78" s="10" t="n"/>
-      <c r="CD78" s="10" t="n"/>
+      <c r="CD78" s="10" t="n">
+        <v>0.75</v>
+      </c>
       <c r="CE78" s="10" t="n"/>
       <c r="CF78" s="10" t="n"/>
       <c r="CG78" s="10" t="n"/>
@@ -31026,277 +31050,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008A7894324D7C3949B4D325554D1FC6DA" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="43dd22c4a0a55be49439aa2cba9a6031">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="be2d32d5-45e4-45f8-8cca-e731efdae529" xmlns:ns3="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="67300191881baa0ec8105967d66c0489" ns2:_="" ns3:_="">
-    <xsd:import namespace="be2d32d5-45e4-45f8-8cca-e731efdae529"/>
-    <xsd:import namespace="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="be2d32d5-45e4-45f8-8cca-e731efdae529" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="10" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="11" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="7ff297e6-98dc-4a77-8782-4199b303df17" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="17" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="20" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="21" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="22" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceBillingMetadata" ma:index="23" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{433bb87c-b111-4230-a796-99831eb60517}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithUsers" ma:index="18" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="19" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="be2d32d5-45e4-45f8-8cca-e731efdae529">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{61F6C236-D8BF-44C7-9186-EFFB515641AA}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{833117D3-06AB-4383-8015-2F0F48E6913B}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{309EB785-FC4A-41B6-BED5-3E2ED4D78668}"/>
 </file>
</xml_diff>

<commit_message>
Update: IWork_2026TimeTracking.xlsx [2026-04-22 17:27 UTC]
</commit_message>
<xml_diff>
--- a/IWork_2026TimeTracking.xlsx
+++ b/IWork_2026TimeTracking.xlsx
@@ -7335,7 +7335,9 @@
         <v>2</v>
       </c>
       <c r="CB9" s="10" t="n"/>
-      <c r="CC9" s="10" t="n"/>
+      <c r="CC9" s="10" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CD9" s="10" t="n"/>
       <c r="CE9" s="10" t="n"/>
       <c r="CF9" s="10" t="n"/>
@@ -7935,7 +7937,9 @@
         <v>1.25</v>
       </c>
       <c r="CB11" s="10" t="n"/>
-      <c r="CC11" s="10" t="n"/>
+      <c r="CC11" s="10" t="n">
+        <v>1.5</v>
+      </c>
       <c r="CD11" s="10" t="n">
         <v>0.25</v>
       </c>
@@ -13865,7 +13869,9 @@
         <v>1.25</v>
       </c>
       <c r="CB32" s="10" t="n"/>
-      <c r="CC32" s="10" t="n"/>
+      <c r="CC32" s="10" t="n">
+        <v>2</v>
+      </c>
       <c r="CD32" s="10" t="n">
         <v>0.75</v>
       </c>
@@ -16874,7 +16880,9 @@
         <v>1.25</v>
       </c>
       <c r="CB43" s="10" t="n"/>
-      <c r="CC43" s="10" t="n"/>
+      <c r="CC43" s="10" t="n">
+        <v>1.25</v>
+      </c>
       <c r="CD43" s="10" t="n">
         <v>1.75</v>
       </c>
@@ -17758,7 +17766,9 @@
       </c>
       <c r="CA46" s="10" t="n"/>
       <c r="CB46" s="10" t="n"/>
-      <c r="CC46" s="10" t="n"/>
+      <c r="CC46" s="10" t="n">
+        <v>2</v>
+      </c>
       <c r="CD46" s="10" t="n">
         <v>0.5</v>
       </c>
@@ -22996,7 +23006,9 @@
       <c r="BZ65" s="13" t="n"/>
       <c r="CA65" s="13" t="n"/>
       <c r="CB65" s="13" t="n"/>
-      <c r="CC65" s="13" t="n"/>
+      <c r="CC65" s="13" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CD65" s="13" t="n">
         <v>0.5</v>
       </c>
@@ -23552,7 +23564,9 @@
         <v>0.5</v>
       </c>
       <c r="CB67" s="10" t="n"/>
-      <c r="CC67" s="10" t="n"/>
+      <c r="CC67" s="10" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CD67" s="10" t="n"/>
       <c r="CE67" s="10" t="n"/>
       <c r="CF67" s="10" t="n"/>
@@ -24939,7 +24953,9 @@
       </c>
       <c r="CA72" s="10" t="n"/>
       <c r="CB72" s="10" t="n"/>
-      <c r="CC72" s="10" t="n"/>
+      <c r="CC72" s="10" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CD72" s="10" t="n">
         <v>0.75</v>
       </c>
@@ -26642,7 +26658,9 @@
         <v>0.25</v>
       </c>
       <c r="CB78" s="10" t="n"/>
-      <c r="CC78" s="10" t="n"/>
+      <c r="CC78" s="10" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CD78" s="10" t="n">
         <v>0.75</v>
       </c>

</xml_diff>

<commit_message>
Update: IWork_2026TimeTracking.xlsx [2026-04-22 17:28 UTC]
</commit_message>
<xml_diff>
--- a/IWork_2026TimeTracking.xlsx
+++ b/IWork_2026TimeTracking.xlsx
@@ -7334,7 +7334,9 @@
       <c r="CA9" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="CB9" s="10" t="n"/>
+      <c r="CB9" s="10" t="n">
+        <v>2.25</v>
+      </c>
       <c r="CC9" s="10" t="n">
         <v>0.5</v>
       </c>
@@ -7936,7 +7938,9 @@
       <c r="CA11" s="10" t="n">
         <v>1.25</v>
       </c>
-      <c r="CB11" s="10" t="n"/>
+      <c r="CB11" s="10" t="n">
+        <v>1.25</v>
+      </c>
       <c r="CC11" s="10" t="n">
         <v>1.5</v>
       </c>
@@ -8218,7 +8222,9 @@
       <c r="BY12" s="10" t="n"/>
       <c r="BZ12" s="10" t="n"/>
       <c r="CA12" s="10" t="n"/>
-      <c r="CB12" s="10" t="n"/>
+      <c r="CB12" s="10" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CC12" s="10" t="n"/>
       <c r="CD12" s="10" t="n"/>
       <c r="CE12" s="10" t="n"/>
@@ -10292,7 +10298,9 @@
         <v>0.75</v>
       </c>
       <c r="CA19" s="10" t="n"/>
-      <c r="CB19" s="10" t="n"/>
+      <c r="CB19" s="10" t="n">
+        <v>1.25</v>
+      </c>
       <c r="CC19" s="10" t="n"/>
       <c r="CD19" s="10" t="n"/>
       <c r="CE19" s="10" t="n"/>
@@ -10580,7 +10588,9 @@
       <c r="CA20" s="10" t="n">
         <v>0.5</v>
       </c>
-      <c r="CB20" s="10" t="n"/>
+      <c r="CB20" s="10" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CC20" s="10" t="n"/>
       <c r="CD20" s="10" t="n"/>
       <c r="CE20" s="10" t="n"/>
@@ -16879,7 +16889,9 @@
       <c r="CA43" s="10" t="n">
         <v>1.25</v>
       </c>
-      <c r="CB43" s="10" t="n"/>
+      <c r="CB43" s="10" t="n">
+        <v>2.75</v>
+      </c>
       <c r="CC43" s="10" t="n">
         <v>1.25</v>
       </c>
@@ -25236,7 +25248,9 @@
       <c r="BY73" s="10" t="n"/>
       <c r="BZ73" s="10" t="n"/>
       <c r="CA73" s="10" t="n"/>
-      <c r="CB73" s="10" t="n"/>
+      <c r="CB73" s="10" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CC73" s="10" t="n"/>
       <c r="CD73" s="10" t="n"/>
       <c r="CE73" s="10" t="n"/>

</xml_diff>

<commit_message>
Update: IWork_2026TimeTracking.xlsx [2026-04-22 17:29 UTC]
</commit_message>
<xml_diff>
--- a/IWork_2026TimeTracking.xlsx
+++ b/IWork_2026TimeTracking.xlsx
@@ -8226,7 +8226,9 @@
         <v>0.5</v>
       </c>
       <c r="CC12" s="10" t="n"/>
-      <c r="CD12" s="10" t="n"/>
+      <c r="CD12" s="10" t="n">
+        <v>1.5</v>
+      </c>
       <c r="CE12" s="10" t="n"/>
       <c r="CF12" s="10" t="n"/>
       <c r="CG12" s="10" t="n"/>
@@ -8506,9 +8508,7 @@
       <c r="CA13" s="10" t="n"/>
       <c r="CB13" s="10" t="n"/>
       <c r="CC13" s="10" t="n"/>
-      <c r="CD13" s="10" t="n">
-        <v>1.5</v>
-      </c>
+      <c r="CD13" s="10" t="n"/>
       <c r="CE13" s="10" t="n"/>
       <c r="CF13" s="10" t="n"/>
       <c r="CG13" s="10" t="n"/>

</xml_diff>

<commit_message>
Update: IWork_2026TimeTracking.xlsx [2026-04-23 20:16 UTC]
</commit_message>
<xml_diff>
--- a/IWork_2026TimeTracking.xlsx
+++ b/IWork_2026TimeTracking.xlsx
@@ -7341,7 +7341,9 @@
         <v>0.5</v>
       </c>
       <c r="CD9" s="10" t="n"/>
-      <c r="CE9" s="10" t="n"/>
+      <c r="CE9" s="10" t="n">
+        <v>0.75</v>
+      </c>
       <c r="CF9" s="10" t="n"/>
       <c r="CG9" s="10" t="n"/>
       <c r="CH9" s="10" t="n"/>
@@ -7947,7 +7949,9 @@
       <c r="CD11" s="10" t="n">
         <v>0.25</v>
       </c>
-      <c r="CE11" s="10" t="n"/>
+      <c r="CE11" s="10" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CF11" s="10" t="n"/>
       <c r="CG11" s="10" t="n"/>
       <c r="CH11" s="10" t="n"/>
@@ -8229,7 +8233,9 @@
       <c r="CD12" s="10" t="n">
         <v>1.5</v>
       </c>
-      <c r="CE12" s="10" t="n"/>
+      <c r="CE12" s="10" t="n">
+        <v>2</v>
+      </c>
       <c r="CF12" s="10" t="n"/>
       <c r="CG12" s="10" t="n"/>
       <c r="CH12" s="10" t="n"/>
@@ -9085,7 +9091,9 @@
       <c r="CB15" s="10" t="n"/>
       <c r="CC15" s="10" t="n"/>
       <c r="CD15" s="10" t="n"/>
-      <c r="CE15" s="10" t="n"/>
+      <c r="CE15" s="10" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CF15" s="10" t="n"/>
       <c r="CG15" s="10" t="n"/>
       <c r="CH15" s="10" t="n"/>
@@ -10303,7 +10311,9 @@
       </c>
       <c r="CC19" s="10" t="n"/>
       <c r="CD19" s="10" t="n"/>
-      <c r="CE19" s="10" t="n"/>
+      <c r="CE19" s="10" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CF19" s="10" t="n"/>
       <c r="CG19" s="10" t="n"/>
       <c r="CH19" s="10" t="n"/>
@@ -10593,7 +10603,9 @@
       </c>
       <c r="CC20" s="10" t="n"/>
       <c r="CD20" s="10" t="n"/>
-      <c r="CE20" s="10" t="n"/>
+      <c r="CE20" s="10" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CF20" s="10" t="n"/>
       <c r="CG20" s="10" t="n"/>
       <c r="CH20" s="10" t="n"/>
@@ -13885,7 +13897,9 @@
       <c r="CD32" s="10" t="n">
         <v>0.75</v>
       </c>
-      <c r="CE32" s="10" t="n"/>
+      <c r="CE32" s="10" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CF32" s="10" t="n"/>
       <c r="CG32" s="10" t="n"/>
       <c r="CH32" s="10" t="n"/>
@@ -16898,7 +16912,9 @@
       <c r="CD43" s="10" t="n">
         <v>1.75</v>
       </c>
-      <c r="CE43" s="10" t="n"/>
+      <c r="CE43" s="10" t="n">
+        <v>0.75</v>
+      </c>
       <c r="CF43" s="10" t="n"/>
       <c r="CG43" s="10" t="n"/>
       <c r="CH43" s="10" t="n"/>
@@ -18935,7 +18951,9 @@
       <c r="CD50" s="10" t="n">
         <v>0.25</v>
       </c>
-      <c r="CE50" s="10" t="n"/>
+      <c r="CE50" s="10" t="n">
+        <v>0.75</v>
+      </c>
       <c r="CF50" s="10" t="n"/>
       <c r="CG50" s="10" t="n"/>
       <c r="CH50" s="10" t="n"/>
@@ -23024,7 +23042,9 @@
       <c r="CD65" s="13" t="n">
         <v>0.5</v>
       </c>
-      <c r="CE65" s="13" t="n"/>
+      <c r="CE65" s="13" t="n">
+        <v>1.25</v>
+      </c>
       <c r="CF65" s="13" t="n"/>
       <c r="CG65" s="13" t="n"/>
       <c r="CH65" s="13" t="n"/>
@@ -23580,7 +23600,9 @@
         <v>0.5</v>
       </c>
       <c r="CD67" s="10" t="n"/>
-      <c r="CE67" s="10" t="n"/>
+      <c r="CE67" s="10" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CF67" s="10" t="n"/>
       <c r="CG67" s="10" t="n"/>
       <c r="CH67" s="10" t="n"/>
@@ -25253,7 +25275,9 @@
       </c>
       <c r="CC73" s="10" t="n"/>
       <c r="CD73" s="10" t="n"/>
-      <c r="CE73" s="10" t="n"/>
+      <c r="CE73" s="10" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CF73" s="10" t="n"/>
       <c r="CG73" s="10" t="n"/>
       <c r="CH73" s="10" t="n"/>

</xml_diff>

<commit_message>
Update: IWork_2026TimeTracking.xlsx [2026-04-28 22:39 UTC]
</commit_message>
<xml_diff>
--- a/IWork_2026TimeTracking.xlsx
+++ b/IWork_2026TimeTracking.xlsx
@@ -7344,7 +7344,9 @@
       <c r="CE9" s="10" t="n">
         <v>0.75</v>
       </c>
-      <c r="CF9" s="10" t="n"/>
+      <c r="CF9" s="10" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CG9" s="10" t="n"/>
       <c r="CH9" s="10" t="n"/>
       <c r="CI9" s="10" t="n"/>
@@ -8236,7 +8238,9 @@
       <c r="CE12" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="CF12" s="10" t="n"/>
+      <c r="CF12" s="10" t="n">
+        <v>1.5</v>
+      </c>
       <c r="CG12" s="10" t="n"/>
       <c r="CH12" s="10" t="n"/>
       <c r="CI12" s="10" t="n"/>
@@ -9094,7 +9098,9 @@
       <c r="CE15" s="10" t="n">
         <v>0.5</v>
       </c>
-      <c r="CF15" s="10" t="n"/>
+      <c r="CF15" s="10" t="n">
+        <v>1</v>
+      </c>
       <c r="CG15" s="10" t="n"/>
       <c r="CH15" s="10" t="n"/>
       <c r="CI15" s="10" t="n"/>
@@ -16915,7 +16921,9 @@
       <c r="CE43" s="10" t="n">
         <v>0.75</v>
       </c>
-      <c r="CF43" s="10" t="n"/>
+      <c r="CF43" s="10" t="n">
+        <v>3.75</v>
+      </c>
       <c r="CG43" s="10" t="n"/>
       <c r="CH43" s="10" t="n"/>
       <c r="CI43" s="10" t="n"/>
@@ -17801,7 +17809,9 @@
         <v>0.5</v>
       </c>
       <c r="CE46" s="10" t="n"/>
-      <c r="CF46" s="10" t="n"/>
+      <c r="CF46" s="10" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CG46" s="10" t="n"/>
       <c r="CH46" s="10" t="n"/>
       <c r="CI46" s="10" t="n"/>
@@ -23045,7 +23055,9 @@
       <c r="CE65" s="13" t="n">
         <v>1.25</v>
       </c>
-      <c r="CF65" s="13" t="n"/>
+      <c r="CF65" s="13" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CG65" s="13" t="n"/>
       <c r="CH65" s="13" t="n"/>
       <c r="CI65" s="13" t="n"/>
@@ -26385,7 +26397,9 @@
       <c r="CC77" s="10" t="n"/>
       <c r="CD77" s="10" t="n"/>
       <c r="CE77" s="10" t="n"/>
-      <c r="CF77" s="10" t="n"/>
+      <c r="CF77" s="10" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CG77" s="10" t="n"/>
       <c r="CH77" s="10" t="n"/>
       <c r="CI77" s="10" t="n"/>

</xml_diff>

<commit_message>
Update: IWork_2026TimeTracking.xlsx [2026-04-28 22:40 UTC]
</commit_message>
<xml_diff>
--- a/IWork_2026TimeTracking.xlsx
+++ b/IWork_2026TimeTracking.xlsx
@@ -7348,7 +7348,9 @@
         <v>0.5</v>
       </c>
       <c r="CG9" s="10" t="n"/>
-      <c r="CH9" s="10" t="n"/>
+      <c r="CH9" s="10" t="n">
+        <v>4.25</v>
+      </c>
       <c r="CI9" s="10" t="n"/>
       <c r="CJ9" s="25" t="n"/>
       <c r="CK9" s="10" t="n"/>
@@ -7956,7 +7958,9 @@
       </c>
       <c r="CF11" s="10" t="n"/>
       <c r="CG11" s="10" t="n"/>
-      <c r="CH11" s="10" t="n"/>
+      <c r="CH11" s="10" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CI11" s="10" t="n"/>
       <c r="CJ11" s="25" t="n"/>
       <c r="CK11" s="10" t="n"/>
@@ -8242,7 +8246,9 @@
         <v>1.5</v>
       </c>
       <c r="CG12" s="10" t="n"/>
-      <c r="CH12" s="10" t="n"/>
+      <c r="CH12" s="10" t="n">
+        <v>1</v>
+      </c>
       <c r="CI12" s="10" t="n"/>
       <c r="CJ12" s="25" t="n"/>
       <c r="CK12" s="10" t="n"/>
@@ -9102,7 +9108,9 @@
         <v>1</v>
       </c>
       <c r="CG15" s="10" t="n"/>
-      <c r="CH15" s="10" t="n"/>
+      <c r="CH15" s="10" t="n">
+        <v>0.75</v>
+      </c>
       <c r="CI15" s="10" t="n"/>
       <c r="CJ15" s="25" t="n"/>
       <c r="CK15" s="10" t="n"/>
@@ -16925,7 +16933,9 @@
         <v>3.75</v>
       </c>
       <c r="CG43" s="10" t="n"/>
-      <c r="CH43" s="10" t="n"/>
+      <c r="CH43" s="10" t="n">
+        <v>1.5</v>
+      </c>
       <c r="CI43" s="10" t="n"/>
       <c r="CJ43" s="25" t="n"/>
       <c r="CK43" s="10" t="n"/>

</xml_diff>

<commit_message>
Update: IWork_2026TimeTracking.xlsx [2026-04-28 22:41 UTC]
</commit_message>
<xml_diff>
--- a/IWork_2026TimeTracking.xlsx
+++ b/IWork_2026TimeTracking.xlsx
@@ -7347,7 +7347,9 @@
       <c r="CF9" s="10" t="n">
         <v>0.5</v>
       </c>
-      <c r="CG9" s="10" t="n"/>
+      <c r="CG9" s="10" t="n">
+        <v>0.75</v>
+      </c>
       <c r="CH9" s="10" t="n">
         <v>4.25</v>
       </c>
@@ -7957,7 +7959,9 @@
         <v>0.25</v>
       </c>
       <c r="CF11" s="10" t="n"/>
-      <c r="CG11" s="10" t="n"/>
+      <c r="CG11" s="10" t="n">
+        <v>1.5</v>
+      </c>
       <c r="CH11" s="10" t="n">
         <v>0.5</v>
       </c>
@@ -8245,7 +8249,9 @@
       <c r="CF12" s="10" t="n">
         <v>1.5</v>
       </c>
-      <c r="CG12" s="10" t="n"/>
+      <c r="CG12" s="10" t="n">
+        <v>1.5</v>
+      </c>
       <c r="CH12" s="10" t="n">
         <v>1</v>
       </c>
@@ -9107,7 +9113,9 @@
       <c r="CF15" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="CG15" s="10" t="n"/>
+      <c r="CG15" s="10" t="n">
+        <v>0.75</v>
+      </c>
       <c r="CH15" s="10" t="n">
         <v>0.75</v>
       </c>
@@ -16932,7 +16940,9 @@
       <c r="CF43" s="10" t="n">
         <v>3.75</v>
       </c>
-      <c r="CG43" s="10" t="n"/>
+      <c r="CG43" s="10" t="n">
+        <v>1</v>
+      </c>
       <c r="CH43" s="10" t="n">
         <v>1.5</v>
       </c>
@@ -17822,7 +17832,9 @@
       <c r="CF46" s="10" t="n">
         <v>0.5</v>
       </c>
-      <c r="CG46" s="10" t="n"/>
+      <c r="CG46" s="10" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CH46" s="10" t="n"/>
       <c r="CI46" s="10" t="n"/>
       <c r="CJ46" s="25" t="n"/>
@@ -18975,7 +18987,9 @@
         <v>0.75</v>
       </c>
       <c r="CF50" s="10" t="n"/>
-      <c r="CG50" s="10" t="n"/>
+      <c r="CG50" s="10" t="n">
+        <v>0.75</v>
+      </c>
       <c r="CH50" s="10" t="n"/>
       <c r="CI50" s="10" t="n"/>
       <c r="CJ50" s="25" t="n"/>
@@ -21975,7 +21989,9 @@
       </c>
       <c r="CE61" s="10" t="n"/>
       <c r="CF61" s="10" t="n"/>
-      <c r="CG61" s="10" t="n"/>
+      <c r="CG61" s="10" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CH61" s="10" t="n"/>
       <c r="CI61" s="10" t="n"/>
       <c r="CJ61" s="25" t="n"/>
@@ -23626,7 +23642,9 @@
         <v>0.5</v>
       </c>
       <c r="CF67" s="10" t="n"/>
-      <c r="CG67" s="10" t="n"/>
+      <c r="CG67" s="10" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CH67" s="10" t="n"/>
       <c r="CI67" s="10" t="n"/>
       <c r="CJ67" s="25" t="n"/>
@@ -25579,7 +25597,9 @@
       <c r="CD74" s="10" t="n"/>
       <c r="CE74" s="10" t="n"/>
       <c r="CF74" s="10" t="n"/>
-      <c r="CG74" s="10" t="n"/>
+      <c r="CG74" s="10" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CH74" s="10" t="n"/>
       <c r="CI74" s="10" t="n"/>
       <c r="CJ74" s="25" t="n"/>

</xml_diff>

<commit_message>
Update: IWork_2026TimeTracking.xlsx [2026-05-05 20:56 UTC]
</commit_message>
<xml_diff>
--- a/IWork_2026TimeTracking.xlsx
+++ b/IWork_2026TimeTracking.xlsx
@@ -7357,7 +7357,9 @@
       <c r="CJ9" s="25" t="n"/>
       <c r="CK9" s="10" t="n"/>
       <c r="CL9" s="10" t="n"/>
-      <c r="CM9" s="10" t="n"/>
+      <c r="CM9" s="10" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CN9" s="10" t="n"/>
       <c r="CO9" s="10" t="n"/>
       <c r="CP9" s="10" t="n"/>
@@ -16950,7 +16952,9 @@
       <c r="CJ43" s="25" t="n"/>
       <c r="CK43" s="10" t="n"/>
       <c r="CL43" s="10" t="n"/>
-      <c r="CM43" s="10" t="n"/>
+      <c r="CM43" s="10" t="n">
+        <v>2</v>
+      </c>
       <c r="CN43" s="10" t="n"/>
       <c r="CO43" s="10" t="n"/>
       <c r="CP43" s="10" t="n"/>
@@ -17520,7 +17524,9 @@
       <c r="CJ45" s="25" t="n"/>
       <c r="CK45" s="10" t="n"/>
       <c r="CL45" s="10" t="n"/>
-      <c r="CM45" s="10" t="n"/>
+      <c r="CM45" s="10" t="n">
+        <v>2.5</v>
+      </c>
       <c r="CN45" s="10" t="n"/>
       <c r="CO45" s="10" t="n"/>
       <c r="CP45" s="10" t="n"/>
@@ -18995,7 +19001,9 @@
       <c r="CJ50" s="25" t="n"/>
       <c r="CK50" s="10" t="n"/>
       <c r="CL50" s="10" t="n"/>
-      <c r="CM50" s="10" t="n"/>
+      <c r="CM50" s="10" t="n">
+        <v>2.5</v>
+      </c>
       <c r="CN50" s="10" t="n"/>
       <c r="CO50" s="10" t="n"/>
       <c r="CP50" s="10" t="n"/>
@@ -23090,7 +23098,9 @@
       <c r="CJ65" s="26" t="n"/>
       <c r="CK65" s="13" t="n"/>
       <c r="CL65" s="13" t="n"/>
-      <c r="CM65" s="13" t="n"/>
+      <c r="CM65" s="13" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CN65" s="13" t="n"/>
       <c r="CO65" s="13" t="n"/>
       <c r="CP65" s="13" t="n"/>
@@ -25041,7 +25051,9 @@
       <c r="CJ72" s="25" t="n"/>
       <c r="CK72" s="10" t="n"/>
       <c r="CL72" s="10" t="n"/>
-      <c r="CM72" s="10" t="n"/>
+      <c r="CM72" s="10" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CN72" s="10" t="n"/>
       <c r="CO72" s="10" t="n"/>
       <c r="CP72" s="10" t="n"/>

</xml_diff>

<commit_message>
Update: IWork_2026TimeTracking.xlsx [2026-05-05 20:57 UTC]
</commit_message>
<xml_diff>
--- a/IWork_2026TimeTracking.xlsx
+++ b/IWork_2026TimeTracking.xlsx
@@ -27894,7 +27894,9 @@
       <c r="CH82" s="10" t="n"/>
       <c r="CI82" s="10" t="n"/>
       <c r="CJ82" s="25" t="n"/>
-      <c r="CK82" s="10" t="n"/>
+      <c r="CK82" s="10" t="n">
+        <v>8</v>
+      </c>
       <c r="CL82" s="10" t="n"/>
       <c r="CM82" s="10" t="n"/>
       <c r="CN82" s="10" t="n"/>

</xml_diff>

<commit_message>
Update: IWork_2026TimeTracking.xlsx [2026-05-05 20:58 UTC]
</commit_message>
<xml_diff>
--- a/IWork_2026TimeTracking.xlsx
+++ b/IWork_2026TimeTracking.xlsx
@@ -27315,7 +27315,9 @@
       <c r="CG80" s="10" t="n"/>
       <c r="CH80" s="10" t="n"/>
       <c r="CI80" s="10" t="n"/>
-      <c r="CJ80" s="25" t="n"/>
+      <c r="CJ80" s="25" t="n">
+        <v>5</v>
+      </c>
       <c r="CK80" s="10" t="n"/>
       <c r="CL80" s="10" t="n"/>
       <c r="CM80" s="10" t="n"/>
@@ -27893,7 +27895,9 @@
       <c r="CG82" s="10" t="n"/>
       <c r="CH82" s="10" t="n"/>
       <c r="CI82" s="10" t="n"/>
-      <c r="CJ82" s="25" t="n"/>
+      <c r="CJ82" s="25" t="n">
+        <v>3</v>
+      </c>
       <c r="CK82" s="10" t="n">
         <v>8</v>
       </c>

</xml_diff>

<commit_message>
Update: IWork_2026TimeTracking.xlsx [2026-05-06 18:57 UTC]
</commit_message>
<xml_diff>
--- a/IWork_2026TimeTracking.xlsx
+++ b/IWork_2026TimeTracking.xlsx
@@ -7360,7 +7360,9 @@
       <c r="CM9" s="10" t="n">
         <v>0.25</v>
       </c>
-      <c r="CN9" s="10" t="n"/>
+      <c r="CN9" s="10" t="n">
+        <v>1</v>
+      </c>
       <c r="CO9" s="10" t="n"/>
       <c r="CP9" s="10" t="n"/>
       <c r="CQ9" s="10" t="n"/>
@@ -8262,7 +8264,9 @@
       <c r="CK12" s="10" t="n"/>
       <c r="CL12" s="10" t="n"/>
       <c r="CM12" s="10" t="n"/>
-      <c r="CN12" s="10" t="n"/>
+      <c r="CN12" s="10" t="n">
+        <v>1.5</v>
+      </c>
       <c r="CO12" s="10" t="n"/>
       <c r="CP12" s="10" t="n"/>
       <c r="CQ12" s="10" t="n"/>
@@ -9448,7 +9452,9 @@
       <c r="CK16" s="10" t="n"/>
       <c r="CL16" s="10" t="n"/>
       <c r="CM16" s="10" t="n"/>
-      <c r="CN16" s="10" t="n"/>
+      <c r="CN16" s="10" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CO16" s="10" t="n"/>
       <c r="CP16" s="10" t="n"/>
       <c r="CQ16" s="10" t="n"/>
@@ -10346,7 +10352,9 @@
       <c r="CK19" s="10" t="n"/>
       <c r="CL19" s="10" t="n"/>
       <c r="CM19" s="10" t="n"/>
-      <c r="CN19" s="10" t="n"/>
+      <c r="CN19" s="10" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CO19" s="10" t="n"/>
       <c r="CP19" s="10" t="n"/>
       <c r="CQ19" s="10" t="n"/>
@@ -16955,7 +16963,9 @@
       <c r="CM43" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="CN43" s="10" t="n"/>
+      <c r="CN43" s="10" t="n">
+        <v>2.25</v>
+      </c>
       <c r="CO43" s="10" t="n"/>
       <c r="CP43" s="10" t="n"/>
       <c r="CQ43" s="10" t="n"/>
@@ -19004,7 +19014,9 @@
       <c r="CM50" s="10" t="n">
         <v>2.5</v>
       </c>
-      <c r="CN50" s="10" t="n"/>
+      <c r="CN50" s="10" t="n">
+        <v>2.5</v>
+      </c>
       <c r="CO50" s="10" t="n"/>
       <c r="CP50" s="10" t="n"/>
       <c r="CQ50" s="10" t="n"/>

</xml_diff>

<commit_message>
Update: IWork_2026TimeTracking.xlsx [2026-05-13 17:29 UTC]
</commit_message>
<xml_diff>
--- a/IWork_2026TimeTracking.xlsx
+++ b/IWork_2026TimeTracking.xlsx
@@ -7353,7 +7353,9 @@
       <c r="CH9" s="10" t="n">
         <v>4.25</v>
       </c>
-      <c r="CI9" s="10" t="n"/>
+      <c r="CI9" s="10" t="n">
+        <v>1.5</v>
+      </c>
       <c r="CJ9" s="25" t="n"/>
       <c r="CK9" s="10" t="n"/>
       <c r="CL9" s="10" t="n"/>
@@ -8259,7 +8261,9 @@
       <c r="CH12" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="CI12" s="10" t="n"/>
+      <c r="CI12" s="10" t="n">
+        <v>1</v>
+      </c>
       <c r="CJ12" s="25" t="n"/>
       <c r="CK12" s="10" t="n"/>
       <c r="CL12" s="10" t="n"/>
@@ -16956,7 +16960,9 @@
       <c r="CH43" s="10" t="n">
         <v>1.5</v>
       </c>
-      <c r="CI43" s="10" t="n"/>
+      <c r="CI43" s="10" t="n">
+        <v>1.5</v>
+      </c>
       <c r="CJ43" s="25" t="n"/>
       <c r="CK43" s="10" t="n"/>
       <c r="CL43" s="10" t="n"/>
@@ -17852,7 +17858,9 @@
         <v>0.5</v>
       </c>
       <c r="CH46" s="10" t="n"/>
-      <c r="CI46" s="10" t="n"/>
+      <c r="CI46" s="10" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CJ46" s="25" t="n"/>
       <c r="CK46" s="10" t="n"/>
       <c r="CL46" s="10" t="n"/>
@@ -19007,7 +19015,9 @@
         <v>0.75</v>
       </c>
       <c r="CH50" s="10" t="n"/>
-      <c r="CI50" s="10" t="n"/>
+      <c r="CI50" s="10" t="n">
+        <v>2</v>
+      </c>
       <c r="CJ50" s="25" t="n"/>
       <c r="CK50" s="10" t="n"/>
       <c r="CL50" s="10" t="n"/>
@@ -25625,7 +25635,9 @@
         <v>0.5</v>
       </c>
       <c r="CH74" s="10" t="n"/>
-      <c r="CI74" s="10" t="n"/>
+      <c r="CI74" s="10" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CJ74" s="25" t="n"/>
       <c r="CK74" s="10" t="n"/>
       <c r="CL74" s="10" t="n"/>
@@ -26774,7 +26786,9 @@
       <c r="CF78" s="10" t="n"/>
       <c r="CG78" s="10" t="n"/>
       <c r="CH78" s="10" t="n"/>
-      <c r="CI78" s="10" t="n"/>
+      <c r="CI78" s="10" t="n">
+        <v>1</v>
+      </c>
       <c r="CJ78" s="25" t="n"/>
       <c r="CK78" s="10" t="n"/>
       <c r="CL78" s="10" t="n"/>

</xml_diff>

<commit_message>
Update: IWork_2026TimeTracking.xlsx [2026-05-13 17:32 UTC]
</commit_message>
<xml_diff>
--- a/IWork_2026TimeTracking.xlsx
+++ b/IWork_2026TimeTracking.xlsx
@@ -7358,7 +7358,9 @@
       </c>
       <c r="CJ9" s="25" t="n"/>
       <c r="CK9" s="10" t="n"/>
-      <c r="CL9" s="10" t="n"/>
+      <c r="CL9" s="10" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CM9" s="10" t="n">
         <v>0.25</v>
       </c>
@@ -7974,7 +7976,9 @@
       <c r="CI11" s="10" t="n"/>
       <c r="CJ11" s="25" t="n"/>
       <c r="CK11" s="10" t="n"/>
-      <c r="CL11" s="10" t="n"/>
+      <c r="CL11" s="10" t="n">
+        <v>1</v>
+      </c>
       <c r="CM11" s="10" t="n"/>
       <c r="CN11" s="10" t="n"/>
       <c r="CO11" s="10" t="n"/>
@@ -9132,7 +9136,9 @@
       <c r="CI15" s="10" t="n"/>
       <c r="CJ15" s="25" t="n"/>
       <c r="CK15" s="10" t="n"/>
-      <c r="CL15" s="10" t="n"/>
+      <c r="CL15" s="10" t="n">
+        <v>1.5</v>
+      </c>
       <c r="CM15" s="10" t="n"/>
       <c r="CN15" s="10" t="n"/>
       <c r="CO15" s="10" t="n"/>
@@ -16965,7 +16971,9 @@
       </c>
       <c r="CJ43" s="25" t="n"/>
       <c r="CK43" s="10" t="n"/>
-      <c r="CL43" s="10" t="n"/>
+      <c r="CL43" s="10" t="n">
+        <v>1.5</v>
+      </c>
       <c r="CM43" s="10" t="n">
         <v>2</v>
       </c>
@@ -17863,7 +17871,9 @@
       </c>
       <c r="CJ46" s="25" t="n"/>
       <c r="CK46" s="10" t="n"/>
-      <c r="CL46" s="10" t="n"/>
+      <c r="CL46" s="10" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CM46" s="10" t="n"/>
       <c r="CN46" s="10" t="n"/>
       <c r="CO46" s="10" t="n"/>
@@ -19020,7 +19030,9 @@
       </c>
       <c r="CJ50" s="25" t="n"/>
       <c r="CK50" s="10" t="n"/>
-      <c r="CL50" s="10" t="n"/>
+      <c r="CL50" s="10" t="n">
+        <v>1.5</v>
+      </c>
       <c r="CM50" s="10" t="n">
         <v>2.5</v>
       </c>
@@ -20391,7 +20403,9 @@
       <c r="CI55" s="10" t="n"/>
       <c r="CJ55" s="25" t="n"/>
       <c r="CK55" s="10" t="n"/>
-      <c r="CL55" s="10" t="n"/>
+      <c r="CL55" s="10" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CM55" s="10" t="n"/>
       <c r="CN55" s="10" t="n"/>
       <c r="CO55" s="10" t="n"/>
@@ -26791,7 +26805,9 @@
       </c>
       <c r="CJ78" s="25" t="n"/>
       <c r="CK78" s="10" t="n"/>
-      <c r="CL78" s="10" t="n"/>
+      <c r="CL78" s="10" t="n">
+        <v>1.5</v>
+      </c>
       <c r="CM78" s="10" t="n"/>
       <c r="CN78" s="10" t="n"/>
       <c r="CO78" s="10" t="n"/>

</xml_diff>

<commit_message>
Update: IWork_2026TimeTracking.xlsx [2026-05-13 17:34 UTC]
</commit_message>
<xml_diff>
--- a/IWork_2026TimeTracking.xlsx
+++ b/IWork_2026TimeTracking.xlsx
@@ -7367,7 +7367,9 @@
       <c r="CN9" s="10" t="n">
         <v>1.25</v>
       </c>
-      <c r="CO9" s="10" t="n"/>
+      <c r="CO9" s="10" t="n">
+        <v>1</v>
+      </c>
       <c r="CP9" s="10" t="n"/>
       <c r="CQ9" s="10" t="n"/>
       <c r="CR9" s="10" t="n"/>
@@ -8275,7 +8277,9 @@
       <c r="CN12" s="10" t="n">
         <v>1.5</v>
       </c>
-      <c r="CO12" s="10" t="n"/>
+      <c r="CO12" s="10" t="n">
+        <v>0.75</v>
+      </c>
       <c r="CP12" s="10" t="n"/>
       <c r="CQ12" s="10" t="n"/>
       <c r="CR12" s="10" t="n"/>
@@ -16980,7 +16984,9 @@
       <c r="CN43" s="10" t="n">
         <v>2.25</v>
       </c>
-      <c r="CO43" s="10" t="n"/>
+      <c r="CO43" s="10" t="n">
+        <v>2</v>
+      </c>
       <c r="CP43" s="10" t="n"/>
       <c r="CQ43" s="10" t="n"/>
       <c r="CR43" s="10" t="n"/>
@@ -17552,7 +17558,9 @@
         <v>2.5</v>
       </c>
       <c r="CN45" s="10" t="n"/>
-      <c r="CO45" s="10" t="n"/>
+      <c r="CO45" s="10" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CP45" s="10" t="n"/>
       <c r="CQ45" s="10" t="n"/>
       <c r="CR45" s="10" t="n"/>
@@ -19039,7 +19047,9 @@
       <c r="CN50" s="10" t="n">
         <v>2.5</v>
       </c>
-      <c r="CO50" s="10" t="n"/>
+      <c r="CO50" s="10" t="n">
+        <v>2</v>
+      </c>
       <c r="CP50" s="10" t="n"/>
       <c r="CQ50" s="10" t="n"/>
       <c r="CR50" s="10" t="n"/>
@@ -23698,7 +23708,9 @@
       <c r="CL67" s="10" t="n"/>
       <c r="CM67" s="10" t="n"/>
       <c r="CN67" s="10" t="n"/>
-      <c r="CO67" s="10" t="n"/>
+      <c r="CO67" s="10" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CP67" s="10" t="n"/>
       <c r="CQ67" s="10" t="n"/>
       <c r="CR67" s="10" t="n"/>
@@ -26810,7 +26822,9 @@
       </c>
       <c r="CM78" s="10" t="n"/>
       <c r="CN78" s="10" t="n"/>
-      <c r="CO78" s="10" t="n"/>
+      <c r="CO78" s="10" t="n">
+        <v>1.25</v>
+      </c>
       <c r="CP78" s="10" t="n"/>
       <c r="CQ78" s="10" t="n"/>
       <c r="CR78" s="10" t="n"/>

</xml_diff>

<commit_message>
Update: IWork_2026TimeTracking.xlsx [2026-05-13 17:37 UTC]
</commit_message>
<xml_diff>
--- a/IWork_2026TimeTracking.xlsx
+++ b/IWork_2026TimeTracking.xlsx
@@ -7370,7 +7370,9 @@
       <c r="CO9" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="CP9" s="10" t="n"/>
+      <c r="CP9" s="10" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CQ9" s="10" t="n"/>
       <c r="CR9" s="10" t="n"/>
       <c r="CS9" s="10" t="n"/>
@@ -9146,7 +9148,9 @@
       <c r="CM15" s="10" t="n"/>
       <c r="CN15" s="10" t="n"/>
       <c r="CO15" s="10" t="n"/>
-      <c r="CP15" s="10" t="n"/>
+      <c r="CP15" s="10" t="n">
+        <v>1.5</v>
+      </c>
       <c r="CQ15" s="10" t="n"/>
       <c r="CR15" s="10" t="n"/>
       <c r="CS15" s="10" t="n"/>
@@ -10014,7 +10018,9 @@
       <c r="CM18" s="10" t="n"/>
       <c r="CN18" s="10" t="n"/>
       <c r="CO18" s="10" t="n"/>
-      <c r="CP18" s="10" t="n"/>
+      <c r="CP18" s="10" t="n">
+        <v>2</v>
+      </c>
       <c r="CQ18" s="10" t="n"/>
       <c r="CR18" s="10" t="n"/>
       <c r="CS18" s="10" t="n"/>
@@ -16987,7 +16993,9 @@
       <c r="CO43" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="CP43" s="10" t="n"/>
+      <c r="CP43" s="10" t="n">
+        <v>1</v>
+      </c>
       <c r="CQ43" s="10" t="n"/>
       <c r="CR43" s="10" t="n"/>
       <c r="CS43" s="10" t="n"/>
@@ -17885,7 +17893,9 @@
       <c r="CM46" s="10" t="n"/>
       <c r="CN46" s="10" t="n"/>
       <c r="CO46" s="10" t="n"/>
-      <c r="CP46" s="10" t="n"/>
+      <c r="CP46" s="10" t="n">
+        <v>1.5</v>
+      </c>
       <c r="CQ46" s="10" t="n"/>
       <c r="CR46" s="10" t="n"/>
       <c r="CS46" s="10" t="n"/>
@@ -19050,7 +19060,9 @@
       <c r="CO50" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="CP50" s="10" t="n"/>
+      <c r="CP50" s="10" t="n">
+        <v>2.25</v>
+      </c>
       <c r="CQ50" s="10" t="n"/>
       <c r="CR50" s="10" t="n"/>
       <c r="CS50" s="10" t="n"/>
@@ -26825,7 +26837,9 @@
       <c r="CO78" s="10" t="n">
         <v>1.25</v>
       </c>
-      <c r="CP78" s="10" t="n"/>
+      <c r="CP78" s="10" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CQ78" s="10" t="n"/>
       <c r="CR78" s="10" t="n"/>
       <c r="CS78" s="10" t="n"/>

</xml_diff>

<commit_message>
Update: IWork_2026TimeTracking.xlsx [2026-05-13 17:40 UTC]
</commit_message>
<xml_diff>
--- a/IWork_2026TimeTracking.xlsx
+++ b/IWork_2026TimeTracking.xlsx
@@ -7373,7 +7373,9 @@
       <c r="CP9" s="10" t="n">
         <v>0.5</v>
       </c>
-      <c r="CQ9" s="10" t="n"/>
+      <c r="CQ9" s="10" t="n">
+        <v>0.75</v>
+      </c>
       <c r="CR9" s="10" t="n"/>
       <c r="CS9" s="10" t="n"/>
       <c r="CT9" s="10" t="n"/>
@@ -7987,7 +7989,9 @@
       <c r="CN11" s="10" t="n"/>
       <c r="CO11" s="10" t="n"/>
       <c r="CP11" s="10" t="n"/>
-      <c r="CQ11" s="10" t="n"/>
+      <c r="CQ11" s="10" t="n">
+        <v>1.75</v>
+      </c>
       <c r="CR11" s="10" t="n"/>
       <c r="CS11" s="10" t="n"/>
       <c r="CT11" s="10" t="n"/>
@@ -16996,7 +17000,9 @@
       <c r="CP43" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="CQ43" s="10" t="n"/>
+      <c r="CQ43" s="10" t="n">
+        <v>1</v>
+      </c>
       <c r="CR43" s="10" t="n"/>
       <c r="CS43" s="10" t="n"/>
       <c r="CT43" s="10" t="n"/>
@@ -17570,7 +17576,9 @@
         <v>0.5</v>
       </c>
       <c r="CP45" s="10" t="n"/>
-      <c r="CQ45" s="10" t="n"/>
+      <c r="CQ45" s="10" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CR45" s="10" t="n"/>
       <c r="CS45" s="10" t="n"/>
       <c r="CT45" s="10" t="n"/>
@@ -19063,7 +19071,9 @@
       <c r="CP50" s="10" t="n">
         <v>2.25</v>
       </c>
-      <c r="CQ50" s="10" t="n"/>
+      <c r="CQ50" s="10" t="n">
+        <v>3</v>
+      </c>
       <c r="CR50" s="10" t="n"/>
       <c r="CS50" s="10" t="n"/>
       <c r="CT50" s="10" t="n"/>
@@ -26840,7 +26850,9 @@
       <c r="CP78" s="10" t="n">
         <v>0.5</v>
       </c>
-      <c r="CQ78" s="10" t="n"/>
+      <c r="CQ78" s="10" t="n">
+        <v>1.25</v>
+      </c>
       <c r="CR78" s="10" t="n"/>
       <c r="CS78" s="10" t="n"/>
       <c r="CT78" s="10" t="n"/>

</xml_diff>

<commit_message>
Update: IWork_2026TimeTracking.xlsx [2026-05-13 17:42 UTC]
</commit_message>
<xml_diff>
--- a/IWork_2026TimeTracking.xlsx
+++ b/IWork_2026TimeTracking.xlsx
@@ -27412,7 +27412,9 @@
       <c r="CT80" s="10" t="n"/>
       <c r="CU80" s="10" t="n"/>
       <c r="CV80" s="10" t="n"/>
-      <c r="CW80" s="10" t="n"/>
+      <c r="CW80" s="10" t="n">
+        <v>8</v>
+      </c>
       <c r="CX80" s="10" t="n"/>
       <c r="CY80" s="10" t="n"/>
       <c r="CZ80" s="10" t="n"/>

</xml_diff>

<commit_message>
Update: IWork_2026TimeTracking.xlsx [2026-05-15 15:54 UTC]
</commit_message>
<xml_diff>
--- a/IWork_2026TimeTracking.xlsx
+++ b/IWork_2026TimeTracking.xlsx
@@ -7378,7 +7378,9 @@
       </c>
       <c r="CR9" s="10" t="n"/>
       <c r="CS9" s="10" t="n"/>
-      <c r="CT9" s="10" t="n"/>
+      <c r="CT9" s="10" t="n">
+        <v>2</v>
+      </c>
       <c r="CU9" s="10" t="n"/>
       <c r="CV9" s="10" t="n"/>
       <c r="CW9" s="10" t="n"/>
@@ -8290,7 +8292,9 @@
       <c r="CQ12" s="10" t="n"/>
       <c r="CR12" s="10" t="n"/>
       <c r="CS12" s="10" t="n"/>
-      <c r="CT12" s="10" t="n"/>
+      <c r="CT12" s="10" t="n">
+        <v>4</v>
+      </c>
       <c r="CU12" s="10" t="n"/>
       <c r="CV12" s="10" t="n"/>
       <c r="CW12" s="10" t="n"/>
@@ -17581,7 +17585,9 @@
       </c>
       <c r="CR45" s="10" t="n"/>
       <c r="CS45" s="10" t="n"/>
-      <c r="CT45" s="10" t="n"/>
+      <c r="CT45" s="10" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CU45" s="10" t="n"/>
       <c r="CV45" s="10" t="n"/>
       <c r="CW45" s="10" t="n"/>
@@ -19076,7 +19082,9 @@
       </c>
       <c r="CR50" s="10" t="n"/>
       <c r="CS50" s="10" t="n"/>
-      <c r="CT50" s="10" t="n"/>
+      <c r="CT50" s="10" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CU50" s="10" t="n"/>
       <c r="CV50" s="10" t="n"/>
       <c r="CW50" s="10" t="n"/>
@@ -25414,7 +25422,9 @@
       <c r="CQ73" s="10" t="n"/>
       <c r="CR73" s="10" t="n"/>
       <c r="CS73" s="10" t="n"/>
-      <c r="CT73" s="10" t="n"/>
+      <c r="CT73" s="10" t="n">
+        <v>1</v>
+      </c>
       <c r="CU73" s="10" t="n"/>
       <c r="CV73" s="10" t="n"/>
       <c r="CW73" s="10" t="n"/>

</xml_diff>

<commit_message>
Update: IWork_2026TimeTracking.xlsx [2026-06-11 19:53 UTC]
</commit_message>
<xml_diff>
--- a/IWork_2026TimeTracking.xlsx
+++ b/IWork_2026TimeTracking.xlsx
@@ -7400,7 +7400,9 @@
       <c r="DK9" s="10" t="n"/>
       <c r="DL9" s="10" t="n"/>
       <c r="DM9" s="10" t="n"/>
-      <c r="DN9" s="10" t="n"/>
+      <c r="DN9" s="10" t="n">
+        <v>1</v>
+      </c>
       <c r="DO9" s="10" t="n"/>
       <c r="DP9" s="10" t="n"/>
       <c r="DQ9" s="10" t="n"/>
@@ -9182,7 +9184,9 @@
       <c r="DK15" s="10" t="n"/>
       <c r="DL15" s="10" t="n"/>
       <c r="DM15" s="10" t="n"/>
-      <c r="DN15" s="10" t="n"/>
+      <c r="DN15" s="10" t="n">
+        <v>6.75</v>
+      </c>
       <c r="DO15" s="10" t="n"/>
       <c r="DP15" s="10" t="n"/>
       <c r="DQ15" s="10" t="n"/>
@@ -12343,7 +12347,9 @@
       <c r="DK26" s="10" t="n"/>
       <c r="DL26" s="10" t="n"/>
       <c r="DM26" s="10" t="n"/>
-      <c r="DN26" s="10" t="n"/>
+      <c r="DN26" s="10" t="n">
+        <v>0.25</v>
+      </c>
       <c r="DO26" s="10" t="n"/>
       <c r="DP26" s="10" t="n"/>
       <c r="DQ26" s="10" t="n"/>

</xml_diff>

<commit_message>
Update: IWork_2026TimeTracking.xlsx [2026-06-11 19:54 UTC]
</commit_message>
<xml_diff>
--- a/IWork_2026TimeTracking.xlsx
+++ b/IWork_2026TimeTracking.xlsx
@@ -7399,7 +7399,9 @@
       <c r="DJ9" s="10" t="n"/>
       <c r="DK9" s="10" t="n"/>
       <c r="DL9" s="10" t="n"/>
-      <c r="DM9" s="10" t="n"/>
+      <c r="DM9" s="10" t="n">
+        <v>0.75</v>
+      </c>
       <c r="DN9" s="10" t="n">
         <v>1</v>
       </c>
@@ -9183,7 +9185,9 @@
       <c r="DJ15" s="10" t="n"/>
       <c r="DK15" s="10" t="n"/>
       <c r="DL15" s="10" t="n"/>
-      <c r="DM15" s="10" t="n"/>
+      <c r="DM15" s="10" t="n">
+        <v>5</v>
+      </c>
       <c r="DN15" s="10" t="n">
         <v>6.75</v>
       </c>
@@ -22113,7 +22117,9 @@
       <c r="DJ61" s="10" t="n"/>
       <c r="DK61" s="10" t="n"/>
       <c r="DL61" s="10" t="n"/>
-      <c r="DM61" s="10" t="n"/>
+      <c r="DM61" s="10" t="n">
+        <v>0.75</v>
+      </c>
       <c r="DN61" s="10" t="n"/>
       <c r="DO61" s="10" t="n"/>
       <c r="DP61" s="10" t="n"/>
@@ -25163,7 +25169,9 @@
       <c r="DJ72" s="10" t="n"/>
       <c r="DK72" s="10" t="n"/>
       <c r="DL72" s="10" t="n"/>
-      <c r="DM72" s="10" t="n"/>
+      <c r="DM72" s="10" t="n">
+        <v>0.75</v>
+      </c>
       <c r="DN72" s="10" t="n"/>
       <c r="DO72" s="10" t="n"/>
       <c r="DP72" s="10" t="n"/>
@@ -26562,7 +26570,9 @@
       <c r="DJ77" s="10" t="n"/>
       <c r="DK77" s="10" t="n"/>
       <c r="DL77" s="10" t="n"/>
-      <c r="DM77" s="10" t="n"/>
+      <c r="DM77" s="10" t="n">
+        <v>1</v>
+      </c>
       <c r="DN77" s="10" t="n"/>
       <c r="DO77" s="10" t="n"/>
       <c r="DP77" s="10" t="n"/>

</xml_diff>

<commit_message>
Update: IWork_2026TimeTracking.xlsx [2026-06-11 19:57 UTC]
</commit_message>
<xml_diff>
--- a/IWork_2026TimeTracking.xlsx
+++ b/IWork_2026TimeTracking.xlsx
@@ -28026,7 +28026,9 @@
       <c r="CX82" s="10" t="n"/>
       <c r="CY82" s="10" t="n"/>
       <c r="CZ82" s="10" t="n"/>
-      <c r="DA82" s="10" t="n"/>
+      <c r="DA82" s="10" t="n">
+        <v>8</v>
+      </c>
       <c r="DB82" s="10" t="n"/>
       <c r="DC82" s="10" t="n"/>
       <c r="DD82" s="10" t="n"/>

</xml_diff>

<commit_message>
Update: IWork_2026TimeTracking.xlsx [2026-06-11 19:58 UTC]
</commit_message>
<xml_diff>
--- a/IWork_2026TimeTracking.xlsx
+++ b/IWork_2026TimeTracking.xlsx
@@ -17035,7 +17035,9 @@
       <c r="DC43" s="10" t="n"/>
       <c r="DD43" s="10" t="n"/>
       <c r="DE43" s="25" t="n"/>
-      <c r="DF43" s="10" t="n"/>
+      <c r="DF43" s="10" t="n">
+        <v>1.5</v>
+      </c>
       <c r="DG43" s="10" t="n"/>
       <c r="DH43" s="10" t="n"/>
       <c r="DI43" s="10" t="n"/>

</xml_diff>

<commit_message>
Update: IWork_2026TimeTracking.xlsx [2026-07-05 02:02 UTC]
</commit_message>
<xml_diff>
--- a/IWork_2026TimeTracking.xlsx
+++ b/IWork_2026TimeTracking.xlsx
@@ -7426,7 +7426,9 @@
       <c r="EA9" s="25" t="n"/>
       <c r="EB9" s="10" t="n"/>
       <c r="EC9" s="10" t="n"/>
-      <c r="ED9" s="10" t="n"/>
+      <c r="ED9" s="10" t="n">
+        <v>2</v>
+      </c>
       <c r="EE9" s="10" t="n"/>
       <c r="EF9" s="10" t="n"/>
       <c r="EG9" s="10" t="n"/>
@@ -17067,7 +17069,9 @@
       <c r="EA43" s="25" t="n"/>
       <c r="EB43" s="10" t="n"/>
       <c r="EC43" s="10" t="n"/>
-      <c r="ED43" s="10" t="n"/>
+      <c r="ED43" s="10" t="n">
+        <v>3</v>
+      </c>
       <c r="EE43" s="10" t="n"/>
       <c r="EF43" s="10" t="n"/>
       <c r="EG43" s="10" t="n"/>
@@ -26929,7 +26933,9 @@
       <c r="EA78" s="25" t="n"/>
       <c r="EB78" s="10" t="n"/>
       <c r="EC78" s="10" t="n"/>
-      <c r="ED78" s="10" t="n"/>
+      <c r="ED78" s="10" t="n">
+        <v>3</v>
+      </c>
       <c r="EE78" s="10" t="n"/>
       <c r="EF78" s="10" t="n"/>
       <c r="EG78" s="10" t="n"/>

</xml_diff>

<commit_message>
Update: IWork_2026TimeTracking.xlsx [2026-07-05 02:03 UTC]
</commit_message>
<xml_diff>
--- a/IWork_2026TimeTracking.xlsx
+++ b/IWork_2026TimeTracking.xlsx
@@ -20514,7 +20514,9 @@
       <c r="DZ55" s="10" t="n"/>
       <c r="EA55" s="25" t="n"/>
       <c r="EB55" s="10" t="n"/>
-      <c r="EC55" s="10" t="n"/>
+      <c r="EC55" s="10" t="n">
+        <v>1</v>
+      </c>
       <c r="ED55" s="10" t="n"/>
       <c r="EE55" s="10" t="n"/>
       <c r="EF55" s="10" t="n"/>

</xml_diff>

<commit_message>
Update: IWork_2026TimeTracking.xlsx [2026-07-05 02:05 UTC]
</commit_message>
<xml_diff>
--- a/IWork_2026TimeTracking.xlsx
+++ b/IWork_2026TimeTracking.xlsx
@@ -7425,7 +7425,9 @@
       <c r="DZ9" s="10" t="n"/>
       <c r="EA9" s="25" t="n"/>
       <c r="EB9" s="10" t="n"/>
-      <c r="EC9" s="10" t="n"/>
+      <c r="EC9" s="10" t="n">
+        <v>0.5</v>
+      </c>
       <c r="ED9" s="10" t="n"/>
       <c r="EE9" s="10" t="n"/>
       <c r="EF9" s="10" t="n"/>
@@ -8043,7 +8045,9 @@
       <c r="DZ11" s="10" t="n"/>
       <c r="EA11" s="25" t="n"/>
       <c r="EB11" s="10" t="n"/>
-      <c r="EC11" s="10" t="n"/>
+      <c r="EC11" s="10" t="n">
+        <v>1.25</v>
+      </c>
       <c r="ED11" s="10" t="n"/>
       <c r="EE11" s="10" t="n"/>
       <c r="EF11" s="10" t="n"/>
@@ -17066,7 +17070,9 @@
       <c r="DZ43" s="10" t="n"/>
       <c r="EA43" s="25" t="n"/>
       <c r="EB43" s="10" t="n"/>
-      <c r="EC43" s="10" t="n"/>
+      <c r="EC43" s="10" t="n">
+        <v>2</v>
+      </c>
       <c r="ED43" s="10" t="n"/>
       <c r="EE43" s="10" t="n"/>
       <c r="EF43" s="10" t="n"/>
@@ -17644,7 +17650,9 @@
       <c r="DZ45" s="10" t="n"/>
       <c r="EA45" s="25" t="n"/>
       <c r="EB45" s="10" t="n"/>
-      <c r="EC45" s="10" t="n"/>
+      <c r="EC45" s="10" t="n">
+        <v>0.25</v>
+      </c>
       <c r="ED45" s="10" t="n"/>
       <c r="EE45" s="10" t="n"/>
       <c r="EF45" s="10" t="n"/>
@@ -17970,7 +17978,9 @@
       <c r="DZ46" s="10" t="n"/>
       <c r="EA46" s="25" t="n"/>
       <c r="EB46" s="10" t="n"/>
-      <c r="EC46" s="10" t="n"/>
+      <c r="EC46" s="10" t="n">
+        <v>0.5</v>
+      </c>
       <c r="ED46" s="10" t="n"/>
       <c r="EE46" s="10" t="n"/>
       <c r="EF46" s="10" t="n"/>
@@ -18526,7 +18536,9 @@
       <c r="DZ48" s="10" t="n"/>
       <c r="EA48" s="25" t="n"/>
       <c r="EB48" s="10" t="n"/>
-      <c r="EC48" s="10" t="n"/>
+      <c r="EC48" s="10" t="n">
+        <v>0.5</v>
+      </c>
       <c r="ED48" s="10" t="n"/>
       <c r="EE48" s="10" t="n"/>
       <c r="EF48" s="10" t="n"/>
@@ -20510,7 +20522,9 @@
       <c r="DZ55" s="10" t="n"/>
       <c r="EA55" s="25" t="n"/>
       <c r="EB55" s="10" t="n"/>
-      <c r="EC55" s="10" t="n"/>
+      <c r="EC55" s="10" t="n">
+        <v>1</v>
+      </c>
       <c r="ED55" s="10" t="n"/>
       <c r="EE55" s="10" t="n"/>
       <c r="EF55" s="10" t="n"/>
@@ -23514,7 +23528,9 @@
       <c r="DZ66" s="10" t="n"/>
       <c r="EA66" s="25" t="n"/>
       <c r="EB66" s="10" t="n"/>
-      <c r="EC66" s="10" t="n"/>
+      <c r="EC66" s="10" t="n">
+        <v>0.25</v>
+      </c>
       <c r="ED66" s="10" t="n"/>
       <c r="EE66" s="10" t="n"/>
       <c r="EF66" s="10" t="n"/>
@@ -25199,7 +25215,9 @@
       <c r="DZ72" s="10" t="n"/>
       <c r="EA72" s="25" t="n"/>
       <c r="EB72" s="10" t="n"/>
-      <c r="EC72" s="10" t="n"/>
+      <c r="EC72" s="10" t="n">
+        <v>0.75</v>
+      </c>
       <c r="ED72" s="10" t="n"/>
       <c r="EE72" s="10" t="n"/>
       <c r="EF72" s="10" t="n"/>
@@ -26928,7 +26946,9 @@
       <c r="DZ78" s="10" t="n"/>
       <c r="EA78" s="25" t="n"/>
       <c r="EB78" s="10" t="n"/>
-      <c r="EC78" s="10" t="n"/>
+      <c r="EC78" s="10" t="n">
+        <v>1</v>
+      </c>
       <c r="ED78" s="10" t="n"/>
       <c r="EE78" s="10" t="n"/>
       <c r="EF78" s="10" t="n"/>

</xml_diff>

<commit_message>
Update: IWork_2026TimeTracking.xlsx [2026-07-05 02:07 UTC]
</commit_message>
<xml_diff>
--- a/IWork_2026TimeTracking.xlsx
+++ b/IWork_2026TimeTracking.xlsx
@@ -7423,7 +7423,9 @@
       <c r="DX9" s="10" t="n"/>
       <c r="DY9" s="10" t="n"/>
       <c r="DZ9" s="10" t="n"/>
-      <c r="EA9" s="25" t="n"/>
+      <c r="EA9" s="25" t="n">
+        <v>3.25</v>
+      </c>
       <c r="EB9" s="10" t="n"/>
       <c r="EC9" s="10" t="n">
         <v>0.5</v>
@@ -8043,7 +8045,9 @@
       <c r="DX11" s="10" t="n"/>
       <c r="DY11" s="10" t="n"/>
       <c r="DZ11" s="10" t="n"/>
-      <c r="EA11" s="25" t="n"/>
+      <c r="EA11" s="25" t="n">
+        <v>0.25</v>
+      </c>
       <c r="EB11" s="10" t="n"/>
       <c r="EC11" s="10" t="n">
         <v>1.25</v>
@@ -8343,7 +8347,9 @@
       <c r="DX12" s="10" t="n"/>
       <c r="DY12" s="10" t="n"/>
       <c r="DZ12" s="10" t="n"/>
-      <c r="EA12" s="25" t="n"/>
+      <c r="EA12" s="25" t="n">
+        <v>1.75</v>
+      </c>
       <c r="EB12" s="10" t="n"/>
       <c r="EC12" s="10" t="n"/>
       <c r="ED12" s="10" t="n"/>
@@ -9539,7 +9545,9 @@
       <c r="DX16" s="10" t="n"/>
       <c r="DY16" s="10" t="n"/>
       <c r="DZ16" s="10" t="n"/>
-      <c r="EA16" s="25" t="n"/>
+      <c r="EA16" s="25" t="n">
+        <v>0.75</v>
+      </c>
       <c r="EB16" s="10" t="n"/>
       <c r="EC16" s="10" t="n"/>
       <c r="ED16" s="10" t="n"/>
@@ -17068,7 +17076,9 @@
       <c r="DX43" s="10" t="n"/>
       <c r="DY43" s="10" t="n"/>
       <c r="DZ43" s="10" t="n"/>
-      <c r="EA43" s="25" t="n"/>
+      <c r="EA43" s="25" t="n">
+        <v>2.5</v>
+      </c>
       <c r="EB43" s="10" t="n"/>
       <c r="EC43" s="10" t="n">
         <v>2</v>
@@ -19151,7 +19161,9 @@
       <c r="DX50" s="10" t="n"/>
       <c r="DY50" s="10" t="n"/>
       <c r="DZ50" s="10" t="n"/>
-      <c r="EA50" s="25" t="n"/>
+      <c r="EA50" s="25" t="n">
+        <v>0.5</v>
+      </c>
       <c r="EB50" s="10" t="n"/>
       <c r="EC50" s="10" t="n"/>
       <c r="ED50" s="10" t="n"/>
@@ -19423,7 +19435,9 @@
       <c r="DX51" s="10" t="n"/>
       <c r="DY51" s="10" t="n"/>
       <c r="DZ51" s="10" t="n"/>
-      <c r="EA51" s="25" t="n"/>
+      <c r="EA51" s="25" t="n">
+        <v>0.5</v>
+      </c>
       <c r="EB51" s="10" t="n"/>
       <c r="EC51" s="10" t="n"/>
       <c r="ED51" s="10" t="n"/>
@@ -26944,7 +26958,9 @@
       <c r="DX78" s="10" t="n"/>
       <c r="DY78" s="10" t="n"/>
       <c r="DZ78" s="10" t="n"/>
-      <c r="EA78" s="25" t="n"/>
+      <c r="EA78" s="25" t="n">
+        <v>0.5</v>
+      </c>
       <c r="EB78" s="10" t="n"/>
       <c r="EC78" s="10" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
Update: IWork_2026TimeTracking.xlsx [2026-07-05 02:09 UTC]
</commit_message>
<xml_diff>
--- a/IWork_2026TimeTracking.xlsx
+++ b/IWork_2026TimeTracking.xlsx
@@ -7422,7 +7422,9 @@
       <c r="DW9" s="10" t="n"/>
       <c r="DX9" s="10" t="n"/>
       <c r="DY9" s="10" t="n"/>
-      <c r="DZ9" s="10" t="n"/>
+      <c r="DZ9" s="10" t="n">
+        <v>1.5</v>
+      </c>
       <c r="EA9" s="25" t="n">
         <v>3.25</v>
       </c>
@@ -17075,7 +17077,9 @@
       <c r="DW43" s="10" t="n"/>
       <c r="DX43" s="10" t="n"/>
       <c r="DY43" s="10" t="n"/>
-      <c r="DZ43" s="10" t="n"/>
+      <c r="DZ43" s="10" t="n">
+        <v>5</v>
+      </c>
       <c r="EA43" s="25" t="n">
         <v>2.5</v>
       </c>
@@ -17657,7 +17661,9 @@
       <c r="DW45" s="10" t="n"/>
       <c r="DX45" s="10" t="n"/>
       <c r="DY45" s="10" t="n"/>
-      <c r="DZ45" s="10" t="n"/>
+      <c r="DZ45" s="10" t="n">
+        <v>1</v>
+      </c>
       <c r="EA45" s="25" t="n"/>
       <c r="EB45" s="10" t="n"/>
       <c r="EC45" s="10" t="n">
@@ -17985,7 +17991,9 @@
       <c r="DW46" s="10" t="n"/>
       <c r="DX46" s="10" t="n"/>
       <c r="DY46" s="10" t="n"/>
-      <c r="DZ46" s="10" t="n"/>
+      <c r="DZ46" s="10" t="n">
+        <v>1.5</v>
+      </c>
       <c r="EA46" s="25" t="n"/>
       <c r="EB46" s="10" t="n"/>
       <c r="EC46" s="10" t="n">

</xml_diff>